<commit_message>
docs(videos): fix publish field placement and content mismatches across all modules
</commit_message>
<xml_diff>
--- a/docs/videos/video_import_file.xlsx
+++ b/docs/videos/video_import_file.xlsx
@@ -1467,43 +1467,6 @@
 RELATED: [01-account-auth-security.md](./01-account-auth-security.md)
 (2FA), [01-account-auth-security.md](./01-account-auth-security.md)
 (change password)
----
-## Technical reference (source of truth)
-**Screens:** `/register` (Account type selector: business / personal /
-shopping), `/login`, `/forgot-password`, `/onboarding/*`, `/your-tools`
-(personal modules), `/discover` (storefront buyer landing), `/account/profile`
-(profile edit), `/account/security` (tabs: Password, Verification, Linked
-Accounts, Activity)
-**User actions (FE hooks):** `useRegister` (personal / shopping via
-`account_type`) · `useRegisterBusiness` (business + onboarding) · `useLogin` ·
-`useLogout` · `useRequestPasswordReset` · `useResetPassword` ·
-`useSendVerificationCode` · `useVerifyCode` · `useToggleTwoFactor` ·
-`useAccountActivity` · `useInitiateProfileChange` / `useConfirmProfileChange`
-(profile, email, photo - code confirmed) · `useLinkedAccounts` ·
-`useInitiateLinkAccount` / `useConfirmLinkAccount` (link - code confirmed) ·
-`useSwitchAccount` · `useSetPrimary` (set default) ·
-`useInitiateUnlinkAccount` / `useConfirmUnlinkAccount` (unlink - code
-confirmed)
-**API endpoints (BE):** `/auth/register` (one endpoint; `account_type` selects
-business / personal / storefront-buyer) · `/businesses/register` (business
-workspace setup) · `/auth/login` · `/auth/logout` · `/auth/forgot-password` ·
-`/auth/reset-password` · `/auth/verify/send` · `/auth/verify` ·
-`/auth/password/initiate` / `/auth/password/confirm` (change password - code
-confirmed) · `/auth/profile/initiate` / `/auth/profile/confirm` (profile/email/
-photo - code confirmed) · `/auth/two-factor` (toggle) · `/auth/activity`
-(feed) · `/linked-accounts` (list) · `/linked-accounts` (initiate link) ·
-`/linked-accounts/confirm` · `/linked-accounts/{id}/switch` ·
-`/linked-accounts/{id}/set-primary` · `/linked-accounts/{id}/unlink` +
-`/linked-accounts/{id}/unlink/confirm`
-**Your Tools hub (FE):** `PersonalModulesPage` (`/your-tools`) - tool card
-grid via `resolveAccessibleNavGroups` + `usePlanAccessibleModules` (cards only
-for accessible groups, ordered by `TOOL_ORDER`, first six visible then Show
-more), descriptions from `toolDescriptions.ts` (`TOOL_DESCRIPTIONS` personal
-vs business voice), locked-tool cards derived from subscription
-`plan_features` + `getAccessibleModules` (business slugs only), status line
-and gating via `hasSubscriptionAccess` + `STATUS_CONFIG` (trial / active /
-past_due / cancelled / suspended / expired + grace period), card targets are
-`MODULE_DEFAULT_ROUTES` / each group's first sub-route.
 PUBLISHED TITLE: See every sign-in, every change - in one feed.
 SHORT-FORM VARIANT: See every sign-in, every change
 PUBLISHED DESCRIPTION: Review your account activity on Custosell - sign-ins, sign-outs, email verification, 2FA events, password changes, and profile updates, each with the device and IP address. Try free + subscribe #custosell #account #signup #Custosell #SmallBusiness
@@ -1513,7 +1476,44 @@
   - Screen-record clips: the Screen flow steps, trimmed to the script beats
   - Captions / subtitles: full on-screen captions exported as a caption file
   - Brand overlay / watermark: Custosell logo, corner placement
-  - Music: royalty-free background bed, low volume under the voiceover</t>
+  - Music: royalty-free background bed, low volume under the voiceover
+  - ---
+  - ## Technical reference (source of truth)
+  - **Screens:** `/register` (Account type selector: business / personal /
+  - shopping), `/login`, `/forgot-password`, `/onboarding/*`, `/your-tools`
+  - (personal modules), `/discover` (storefront buyer landing), `/account/profile`
+  - (profile edit), `/account/security` (tabs: Password, Verification, Linked
+  - Accounts, Activity)
+  - **User actions (FE hooks):** `useRegister` (personal / shopping via
+  - `account_type`) · `useRegisterBusiness` (business + onboarding) · `useLogin` ·
+  - `useLogout` · `useRequestPasswordReset` · `useResetPassword` ·
+  - `useSendVerificationCode` · `useVerifyCode` · `useToggleTwoFactor` ·
+  - `useAccountActivity` · `useInitiateProfileChange` / `useConfirmProfileChange`
+  - (profile, email, photo - code confirmed) · `useLinkedAccounts` ·
+  - `useInitiateLinkAccount` / `useConfirmLinkAccount` (link - code confirmed) ·
+  - `useSwitchAccount` · `useSetPrimary` (set default) ·
+  - `useInitiateUnlinkAccount` / `useConfirmUnlinkAccount` (unlink - code
+  - confirmed)
+  - **API endpoints (BE):** `/auth/register` (one endpoint; `account_type` selects
+  - business / personal / storefront-buyer) · `/businesses/register` (business
+  - workspace setup) · `/auth/login` · `/auth/logout` · `/auth/forgot-password` ·
+  - `/auth/reset-password` · `/auth/verify/send` · `/auth/verify` ·
+  - `/auth/password/initiate` / `/auth/password/confirm` (change password - code
+  - confirmed) · `/auth/profile/initiate` / `/auth/profile/confirm` (profile/email/
+  - photo - code confirmed) · `/auth/two-factor` (toggle) · `/auth/activity`
+  - (feed) · `/linked-accounts` (list) · `/linked-accounts` (initiate link) ·
+  - `/linked-accounts/confirm` · `/linked-accounts/{id}/switch` ·
+  - `/linked-accounts/{id}/set-primary` · `/linked-accounts/{id}/unlink` +
+  - `/linked-accounts/{id}/unlink/confirm`
+  - **Your Tools hub (FE):** `PersonalModulesPage` (`/your-tools`) - tool card
+  - grid via `resolveAccessibleNavGroups` + `usePlanAccessibleModules` (cards only
+  - for accessible groups, ordered by `TOOL_ORDER`, first six visible then Show
+  - more), descriptions from `toolDescriptions.ts` (`TOOL_DESCRIPTIONS` personal
+  - vs business voice), locked-tool cards derived from subscription
+  - `plan_features` + `getAccessibleModules` (business slugs only), status line
+  - and gating via `hasSubscriptionAccess` + `STATUS_CONFIG` (trial / active /
+  - past_due / cancelled / suspended / expired + grace period), card targets are
+  - `MODULE_DEFAULT_ROUTES` / each group's first sub-route.</t>
         </is>
       </c>
       <c r="D17" s="5" t="n"/>
@@ -2129,46 +2129,6 @@
 DEMO DATA: A business owner account.
 CTA: Try free + subscribe
 RELATED: [17-settings.md](./17-settings.md)
----
-## Technical reference (source of truth)
-**Screens:** `/settings/business` [M] (Profile / Location / Payments / Receipts / Social tabs) ·
-`/settings/tax` [M] (tax profile, EFRIS status, VAT summary) ·
-`/settings/staff` [M] (staff list, add/edit, transfer, transfer history) ·
-`/settings/roles` [M] (role CRUD, system roles protected) ·
-`/settings/locations` [M] (branch CRUD, set default) ·
-`/settings/modules` [M, owner] (module tiles + Estimates/HR depth) ·
-`/settings/data-export` (owner-only export) ·
-`/settings/subscription` and `/settings/sales-channels` covered in [16-subscriptions-billing.md](./16-subscriptions-billing.md) and [14-storefront.md](./14-storefront.md).
-**User actions (FE hooks):** `useBusiness` · `useUpdateBusiness` ·
-`useBusinessExport` · `useInitiateBusinessDelete` · `useConfirmBusinessDelete` ·
-`useBusinessSocialLinks` · `useUpsertBusinessSocialLink` ·
-`useDeleteBusinessSocialLink` · `useVatSummary` · `useEfrisStatus` ·
-`useStaff` · `useCreateStaff` · `useUpdateStaff` · `useAttachStaff` ·
-`useDetachStaff` · `lookupStaffEmail` · `useRoles` · `useCreateRole` ·
-`useUpdateRole` · `useDeleteRole` · `useLocations` · `useCreateLocation` ·
-`useUpdateLocation` · `useSetDefaultLocation` · `useDeleteLocation`.
-**API endpoints (BE):** `GET /businesses/mine` · `PUT /businesses/profile`
-(logo upload uses multipart via `POST ...?_method=PUT`) ·
-`GET /businesses/export?format=json|csv|xlsx` ·
-`POST /businesses/account/initiate` (throttle 3/min) ·
-`POST /businesses/account/confirm` (throttle 10/min) ·
-`GET|POST /business-social-links` · `PUT|DELETE /business-social-links/{id}` ·
-`GET /reports/vat-summary?date_from&amp;date_to&amp;format` ·
-`GET /efris/status` · `GET|POST /users` · `PUT /users/{id}` ·
-`GET /users/lookup?email` · `POST /users/attach` · `POST /users/{id}/detach` ·
-`GET|POST /roles` · `PUT|DELETE /roles/{id}` ·
-`GET|POST /locations` · `PUT|DELETE /locations/{id}` ·
-`POST /locations/{id}/default` · `PUT /auth/profile` (owner module access).
-**Middleware:** business + social-link + staff/role/location management routes
-use `auth:sanctum` + `business.active` + `subscription.active` + `module:settings`;
-`business-social-links` additionally requires `business.owner`; EFRIS status and
-VAT summary require `subscription.active` (no settings gate); `GET /locations`
-reads are open to any active business user, only writes need `module:settings`.
-Delete-account confirm logs the user out and redirects to login.
-**Notable behavior:** business settings, staff, and roles updates can complete
-locally and sync when back online (pending-sync badges); export and delete flows
-are owner-only; personal accounts keep only Profile + Location tabs and skip the
-Danger Zone.
 PUBLISHED TITLE: Your app, your workspaces.
 SHORT-FORM VARIANT: Your app
 PUBLISHED DESCRIPTION: Pick which workspaces the business owner sees on Custosell - hide the modules you don't use and go deeper on Estimates or HR with full access toggles, all from one screen. Try free + subscribe #custosell #settings #businessprofile #tax #Custosell #SmallBusiness
@@ -2178,7 +2138,47 @@
   - Screen-record clips: the Screen flow steps, trimmed to the script beats
   - Captions / subtitles: full on-screen captions exported as a caption file
   - Brand overlay / watermark: Custosell logo, corner placement
-  - Music: royalty-free background bed, low volume under the voiceover</t>
+  - Music: royalty-free background bed, low volume under the voiceover
+  - ---
+  - ## Technical reference (source of truth)
+  - **Screens:** `/settings/business` [M] (Profile / Location / Payments / Receipts / Social tabs) ·
+  - `/settings/tax` [M] (tax profile, EFRIS status, VAT summary) ·
+  - `/settings/staff` [M] (staff list, add/edit, transfer, transfer history) ·
+  - `/settings/roles` [M] (role CRUD, system roles protected) ·
+  - `/settings/locations` [M] (branch CRUD, set default) ·
+  - `/settings/modules` [M, owner] (module tiles + Estimates/HR depth) ·
+  - `/settings/data-export` (owner-only export) ·
+  - `/settings/subscription` and `/settings/sales-channels` covered in [16-subscriptions-billing.md](./16-subscriptions-billing.md) and [14-storefront.md](./14-storefront.md).
+  - **User actions (FE hooks):** `useBusiness` · `useUpdateBusiness` ·
+  - `useBusinessExport` · `useInitiateBusinessDelete` · `useConfirmBusinessDelete` ·
+  - `useBusinessSocialLinks` · `useUpsertBusinessSocialLink` ·
+  - `useDeleteBusinessSocialLink` · `useVatSummary` · `useEfrisStatus` ·
+  - `useStaff` · `useCreateStaff` · `useUpdateStaff` · `useAttachStaff` ·
+  - `useDetachStaff` · `lookupStaffEmail` · `useRoles` · `useCreateRole` ·
+  - `useUpdateRole` · `useDeleteRole` · `useLocations` · `useCreateLocation` ·
+  - `useUpdateLocation` · `useSetDefaultLocation` · `useDeleteLocation`.
+  - **API endpoints (BE):** `GET /businesses/mine` · `PUT /businesses/profile`
+  - (logo upload uses multipart via `POST ...?_method=PUT`) ·
+  - `GET /businesses/export?format=json|csv|xlsx` ·
+  - `POST /businesses/account/initiate` (throttle 3/min) ·
+  - `POST /businesses/account/confirm` (throttle 10/min) ·
+  - `GET|POST /business-social-links` · `PUT|DELETE /business-social-links/{id}` ·
+  - `GET /reports/vat-summary?date_from&amp;date_to&amp;format` ·
+  - `GET /efris/status` · `GET|POST /users` · `PUT /users/{id}` ·
+  - `GET /users/lookup?email` · `POST /users/attach` · `POST /users/{id}/detach` ·
+  - `GET|POST /roles` · `PUT|DELETE /roles/{id}` ·
+  - `GET|POST /locations` · `PUT|DELETE /locations/{id}` ·
+  - `POST /locations/{id}/default` · `PUT /auth/profile` (owner module access).
+  - **Middleware:** business + social-link + staff/role/location management routes
+  - use `auth:sanctum` + `business.active` + `subscription.active` + `module:settings`;
+  - `business-social-links` additionally requires `business.owner`; EFRIS status and
+  - VAT summary require `subscription.active` (no settings gate); `GET /locations`
+  - reads are open to any active business user, only writes need `module:settings`.
+  - Delete-account confirm logs the user out and redirects to login.
+  - **Notable behavior:** business settings, staff, and roles updates can complete
+  - locally and sync when back online (pending-sync badges); export and delete flows
+  - are owner-only; personal accounts keep only Profile + Location tabs and skip the
+  - Danger Zone.</t>
         </is>
       </c>
       <c r="D28" s="5" t="n"/>
@@ -2632,8 +2632,8 @@
 DEMO DATA: A product with a barcode.
 CTA: Try free
 RELATED: [03-sales-pos.md](./03-sales-pos.md)
-PUBLISHED TITLE: Find any product in a second.
-SHORT-FORM VARIANT: Find any product
+PUBLISHED TITLE: SKU and barcode find any product in a second.
+SHORT-FORM VARIANT: SKU. Barcode. Found.
 PUBLISHED DESCRIPTION: Add a SKU and barcode to products so you can search and scan them fast at the till and in the catalog. Try free #custosell #inventory #products #categories #Custosell #SmallBusiness
 TAGS: custosell, inventory, products, categories, sku, barcode, stock, low stock, how to, tutorial, walkthrough, tips
 VIDEO ASSETS:
@@ -3152,8 +3152,8 @@
 DEMO DATA: Products at various stock levels including low and out.
 CTA: Try free
 RELATED: [06-marketplace-purchase-orders.md](./06-marketplace-purchase-orders.md)
-PUBLISHED TITLE: Out of stock before you run out of stock.
-SHORT-FORM VARIANT: Out of stock before you run out of stock.
+PUBLISHED TITLE: Spot low stock before you run out.
+SHORT-FORM VARIANT: Spot low stock before it's gone
 PUBLISHED DESCRIPTION: Read your stock level indicator on Custosell - see what's low, what's out, and what needs restocking at a glance. Try free #custosell #inventory #products #categories #Custosell #SmallBusiness
 TAGS: custosell, inventory, products, categories, sku, barcode, stock, low stock, how to, tutorial, walkthrough, tips
 VIDEO ASSETS:
@@ -3617,26 +3617,6 @@
 DEMO DATA: A disconnected device and an existing catalog.
 CTA: Try free
 RELATED: [21-offline-sync.md](./21-offline-sync.md)
----
-## Technical reference (source of truth)
-**Screens:** `/inventory/overview` [M], `/inventory/products` [M],
-`/inventory/categories`, `/inventory/stock`
-**User actions (FE hooks):** `useProducts` · `useProduct` ·
-`useCreateProduct` · `useUpdateProduct` · `useDeleteProduct` ·
-`useBulkUpdateListing` · `useCategories` · `useCreateCategory` ·
-`useUpdateCategory` · `useDeleteCategory` · `useCreateStockMovement` ·
-`useStockMovements` · `useProductStockMovements` · `useLowStockProducts` ·
-`useLocationStock` · `useStockTransfer` · `useInventoryOverview` ·
-`useUpdateSupplyListing` · `useUpdateStorefrontListing` ·
-`useUploadProductImage`
-**API endpoints (BE):** `/products` CRUD · `/products/low-stock` ·
-`/products/stock/{locationId}` · `/products/import-template` ·
-`/products/import` · `/products/export` · `/products/{id}/stock-movements` ·
-`/products/bulk-delete` · `/products/bulk-listing` ·
-`/products/{id}/supply-listing` · `/products/{id}/storefront-listing` ·
-`/products/{id}/image` · `/categories` CRUD · `/stock-movements` CRUD +
-`/stock-movements/bulk-delete` + `/stock-movements/transfer` ·
-`/inventory/overview`
 PUBLISHED TITLE: Keep building your catalog without internet.
 SHORT-FORM VARIANT: Keep building your catalog without internet.
 PUBLISHED DESCRIPTION: Create, edit, and adjust products even when offline - Custosell queues the changes and syncs them when you're back online. Try free #custosell #inventory #products #categories #Custosell #SmallBusiness
@@ -3646,7 +3626,27 @@
   - Screen-record clips: the Screen flow steps, trimmed to the script beats
   - Captions / subtitles: full on-screen captions exported as a caption file
   - Brand overlay / watermark: Custosell logo, corner placement
-  - Music: royalty-free background bed, low volume under the voiceover</t>
+  - Music: royalty-free background bed, low volume under the voiceover
+  - ---
+  - ## Technical reference (source of truth)
+  - **Screens:** `/inventory/overview` [M], `/inventory/products` [M],
+  - `/inventory/categories`, `/inventory/stock`
+  - **User actions (FE hooks):** `useProducts` · `useProduct` ·
+  - `useCreateProduct` · `useUpdateProduct` · `useDeleteProduct` ·
+  - `useBulkUpdateListing` · `useCategories` · `useCreateCategory` ·
+  - `useUpdateCategory` · `useDeleteCategory` · `useCreateStockMovement` ·
+  - `useStockMovements` · `useProductStockMovements` · `useLowStockProducts` ·
+  - `useLocationStock` · `useStockTransfer` · `useInventoryOverview` ·
+  - `useUpdateSupplyListing` · `useUpdateStorefrontListing` ·
+  - `useUploadProductImage`
+  - **API endpoints (BE):** `/products` CRUD · `/products/low-stock` ·
+  - `/products/stock/{locationId}` · `/products/import-template` ·
+  - `/products/import` · `/products/export` · `/products/{id}/stock-movements` ·
+  - `/products/bulk-delete` · `/products/bulk-listing` ·
+  - `/products/{id}/supply-listing` · `/products/{id}/storefront-listing` ·
+  - `/products/{id}/image` · `/categories` CRUD · `/stock-movements` CRUD +
+  - `/stock-movements/bulk-delete` + `/stock-movements/transfer` ·
+  - `/inventory/overview`</t>
         </is>
       </c>
       <c r="D53" s="5" t="n"/>
@@ -5623,32 +5623,6 @@
 DEMO DATA: A synced sale to refund and offline mode enabled.
 CTA: Try free
 RELATED: [21-offline-sync.md](./21-offline-sync.md)
----
-## Technical reference (source of truth)
-**Screens:** `/sales` -&gt; `/sales/new` [M] (CheckoutStepper: Items -&gt; Payment;
-SaleItemsStep: search/scan, cart, tier toggles, line discounts, Hold Order,
-Take Order, Generate Invoice, Manage Orders/Invoices) · `/sales/orders` [M]
-(status tabs Open/Completed/Invoiced/Cancelled, Online filter, search, branch
-filter, Delivery popover, Resume/Update/Rename/Cancel, invoice from sale) ·
-`/sales/history` [M] (search by receipt, branch/status filters, Select All,
-bulk delete, fiscal status, invoice/email/payments row actions, net + refunds
-summary) · `/sales/refunds` [M] (find by receipt, per-item refund quantities,
-refund total + max-refundable + net remaining, bulk delete) ·
-`/sales/my-shift` [M] (shift-scoped receipts, stat cards, shift summary) ·
-`/invoices`, `/invoices/supplier`
-**User actions (FE hooks):** `useCreateSale` (checkout, online or offline) ·
-`useRefund` (item-level refund, offline-aware) · `useRecordSalePayment`
-(collect balance) · `useAssignSaleCustomer` · `useResolveCustomerContact`
-(walk-in customer at checkout) · `useEmailSaleReceipt` (email receipt) ·
-`useSale` / `useDailySales` / `useShiftSales` · `useCreateOrder` /
-`useUpdateOrder` / `useCancelOrder` (hold/draft, offline-aware) ·
-`useOpenOrders` / `useOrders` (polling list) · `useCreateInvoice` /
-`useSendInvoice` / `useRecordPayment` / `useEmailInvoice` / `viewInvoicePdf`
-**API endpoints (BE):** `/sales` CRUD · `/sales/daily` · `/sales/by-shift/{id}`
-· `/sales/batch` (offline sync) · `/sales/bulk-delete` · `/sales/{id}/refund` ·
-`/sales/{id}/payment` · `/sales/{id}/customer` · `/sales/{id}/pdf` ·
-`/sales/{id}/email` · `/orders` (index/store) · `/orders/{id}` (show/update) ·
-`/orders/{id}/cancel` · `/invoices` CRUD + `/send` `/payment` `/email` `/pdf`
 PUBLISHED TITLE: Refund offline? Saved - and synced when you're back.
 SHORT-FORM VARIANT: Refund offline? Saved
 PUBLISHED DESCRIPTION: Process a refund with no internet on Custosell. It saves locally and syncs when you reconnect; sales that haven't synced yet are protected from being refunded early. Try free #custosell #pos #pointofsale #sell #Custosell #SmallBusiness
@@ -5658,7 +5632,33 @@
   - Screen-record clips: the Screen flow steps, trimmed to the script beats
   - Captions / subtitles: full on-screen captions exported as a caption file
   - Brand overlay / watermark: Custosell logo, corner placement
-  - Music: royalty-free background bed, low volume under the voiceover</t>
+  - Music: royalty-free background bed, low volume under the voiceover
+  - ---
+  - ## Technical reference (source of truth)
+  - **Screens:** `/sales` -&gt; `/sales/new` [M] (CheckoutStepper: Items -&gt; Payment;
+  - SaleItemsStep: search/scan, cart, tier toggles, line discounts, Hold Order,
+  - Take Order, Generate Invoice, Manage Orders/Invoices) · `/sales/orders` [M]
+  - (status tabs Open/Completed/Invoiced/Cancelled, Online filter, search, branch
+  - filter, Delivery popover, Resume/Update/Rename/Cancel, invoice from sale) ·
+  - `/sales/history` [M] (search by receipt, branch/status filters, Select All,
+  - bulk delete, fiscal status, invoice/email/payments row actions, net + refunds
+  - summary) · `/sales/refunds` [M] (find by receipt, per-item refund quantities,
+  - refund total + max-refundable + net remaining, bulk delete) ·
+  - `/sales/my-shift` [M] (shift-scoped receipts, stat cards, shift summary) ·
+  - `/invoices`, `/invoices/supplier`
+  - **User actions (FE hooks):** `useCreateSale` (checkout, online or offline) ·
+  - `useRefund` (item-level refund, offline-aware) · `useRecordSalePayment`
+  - (collect balance) · `useAssignSaleCustomer` · `useResolveCustomerContact`
+  - (walk-in customer at checkout) · `useEmailSaleReceipt` (email receipt) ·
+  - `useSale` / `useDailySales` / `useShiftSales` · `useCreateOrder` /
+  - `useUpdateOrder` / `useCancelOrder` (hold/draft, offline-aware) ·
+  - `useOpenOrders` / `useOrders` (polling list) · `useCreateInvoice` /
+  - `useSendInvoice` / `useRecordPayment` / `useEmailInvoice` / `viewInvoicePdf`
+  - **API endpoints (BE):** `/sales` CRUD · `/sales/daily` · `/sales/by-shift/{id}`
+  - · `/sales/batch` (offline sync) · `/sales/bulk-delete` · `/sales/{id}/refund` ·
+  - `/sales/{id}/payment` · `/sales/{id}/customer` · `/sales/{id}/pdf` ·
+  - `/sales/{id}/email` · `/orders` (index/store) · `/orders/{id}` (show/update) ·
+  - `/orders/{id}/cancel` · `/invoices` CRUD + `/send` `/payment` `/email` `/pdf`</t>
         </is>
       </c>
       <c r="D87" s="5" t="n"/>
@@ -6798,27 +6798,6 @@
 CTA: Try free
 RELATED: [02-dashboard-reports.md](./02-dashboard-reports.md)
 (branch card)
----
-## Technical reference (source of truth)
-**Screens:** `/dashboard` [M] (5 KPI cards, 7-Day Net Sales Trend chart, Low
-Stock Alerts, Recent Activity, Branch Performance card, QuickReports download
-panel, VAT today section, Today's Expenses by Category pie)
-**Report catalog (QuickReports panel, 10 types):** Business Summary (P&amp;L
-snapshot) · Daily Sales · Sales Trend · Product Performance · Shift
-Reconciliation · Expenses · VAT Summary · Inventory (snapshot) · Branch
-Performance (on-screen table) · Payment Breakdown. Each supports date presets
-(Today / This week / This month / This year / Custom) and, where applicable,
-Sales Person + Shift filters, plus PDF / XLSX / CSV export formats.
-**User actions (FE hooks):** `useDashboardSummary` (KPIs + trend + low stock +
-recent sales + today VAT) · `useExpenseSummary` (expense pie) ·
-`useBranchPerformance` (branch card + full report) · `useReportDownload`
-(QuickReports download, blob handling) · `useBusinessTaxSettings` (VAT
-section)
-**API endpoints (BE):** `/dashboard/summary` · `/reports/business-summary` ·
-`/reports/daily-sales` · `/reports/sales-trend` · `/reports/product-performance`
-· `/reports/shift-reconciliation` · `/reports/shift-close` ·
-`/reports/expenses` · `/reports/vat-summary` · `/reports/inventory` ·
-`/reports/payment-breakdown` · `/reports/branch-performance`
 PUBLISHED TITLE: Every branch gross, expenses, net, transactions, share.
 SHORT-FORM VARIANT: Every branch: gross, expenses, net, transactions
 PUBLISHED DESCRIPTION: Open the full Branch Performance report on Custosell - per branch gross, expenses, net sales, transactions, and market share - for any period, right on screen. Try free #custosell #dashboard #reports #salesreport #Custosell #SmallBusiness
@@ -6828,7 +6807,28 @@
   - Screen-record clips: the Screen flow steps, trimmed to the script beats
   - Captions / subtitles: full on-screen captions exported as a caption file
   - Brand overlay / watermark: Custosell logo, corner placement
-  - Music: royalty-free background bed, low volume under the voiceover</t>
+  - Music: royalty-free background bed, low volume under the voiceover
+  - ---
+  - ## Technical reference (source of truth)
+  - **Screens:** `/dashboard` [M] (5 KPI cards, 7-Day Net Sales Trend chart, Low
+  - Stock Alerts, Recent Activity, Branch Performance card, QuickReports download
+  - panel, VAT today section, Today's Expenses by Category pie)
+  - **Report catalog (QuickReports panel, 10 types):** Business Summary (P&amp;L
+  - snapshot) · Daily Sales · Sales Trend · Product Performance · Shift
+  - Reconciliation · Expenses · VAT Summary · Inventory (snapshot) · Branch
+  - Performance (on-screen table) · Payment Breakdown. Each supports date presets
+  - (Today / This week / This month / This year / Custom) and, where applicable,
+  - Sales Person + Shift filters, plus PDF / XLSX / CSV export formats.
+  - **User actions (FE hooks):** `useDashboardSummary` (KPIs + trend + low stock +
+  - recent sales + today VAT) · `useExpenseSummary` (expense pie) ·
+  - `useBranchPerformance` (branch card + full report) · `useReportDownload`
+  - (QuickReports download, blob handling) · `useBusinessTaxSettings` (VAT
+  - section)
+  - **API endpoints (BE):** `/dashboard/summary` · `/reports/business-summary` ·
+  - `/reports/daily-sales` · `/reports/sales-trend` · `/reports/product-performance`
+  - · `/reports/shift-reconciliation` · `/reports/shift-close` ·
+  - `/reports/expenses` · `/reports/vat-summary` · `/reports/inventory` ·
+  - `/reports/payment-breakdown` · `/reports/branch-performance`</t>
         </is>
       </c>
       <c r="D107" s="5" t="n"/>
@@ -7168,7 +7168,7 @@
 ON-SCREEN TEXT / CAPTIONS:
   - "One page, whole shift"
   - "Print or PDF"
-DEMO DATA: An open shift with sales, refunds, expenses, and VAT.
+DEMO DATA: A closed shift with sales, refunds, expenses, and VAT.
 CTA: Try free
 RELATED: [04-shifts.md](./04-shifts.md) (close your shift),
 [02-dashboard-reports.md](./02-dashboard-reports.md) (shift report)
@@ -7406,26 +7406,6 @@
 CTA: Try free
 RELATED: [21-offline-sync.md](./21-offline-sync.md),
 [03-sales-pos.md](./03-sales-pos.md) (sell offline)
----
-## Technical reference (source of truth)
-**Screens:** `/sales/my-shift` [M] (Start Shift, stat cards, Shift Summary,
-Shift Progress chart, Shift Receipts, Shift Expenses, Past Shift Net Sales
-chart, Shift History table, Shift Report preview, Balance Shift, Record
-Expense, End Shift) · `/sales/history` (per-shift sales via filters) ·
-`/sales/refunds` (per shift)
-**User actions (FE hooks):** `useActiveShift` / `useShifts` / `useShiftSales`
-(/sales/by-shift) / `useShiftPayments` (/shifts/{id}/payments) /
-`useShiftExpenses` (/expenses?shift_id=) · `useClockIn` (start shift) ·
-`useClockOut` (end shift + totals: total_sales, total_cash,
-total_mobile_money, total_card, counted_cash) · `useUpdateShiftOpeningBalance`
-(opening_balance) · `useUpdateShiftBalance` (opening_balance + counted_cash) ·
-`useEndShiftAction` (totals math + logout) · `buildShiftCloseReportData` /
-`canDownloadShiftClosePdf` / `downloadShiftClosePdf` (report + PDF)
-**API endpoints (BE):** `/shifts` CRUD (POST = clock in, PUT = opening balance
-/ counted cash / clock out + close) · `/shifts/active` (current shift) ·
-`/shifts/{id}/payments` (shift payments) · `/sales/by-shift/{id}` (shift
-sales) · `/expenses?shift_id={id}` (shift expenses) · `/sales/daily` (day
-rollup per shift)
 PUBLISHED TITLE: Clock in, sell, and close - even with no internet.
 SHORT-FORM VARIANT: Clock in, sell, and close
 PUBLISHED DESCRIPTION: Open, run, and close a shift with no internet on Custosell. Shift changes save locally and sync when you reconnect - the drawer stays accountable the whole time. Try free #custosell #shift #openingbalance #cashdrawer #Custosell #SmallBusiness
@@ -7435,7 +7415,27 @@
   - Screen-record clips: the Screen flow steps, trimmed to the script beats
   - Captions / subtitles: full on-screen captions exported as a caption file
   - Brand overlay / watermark: Custosell logo, corner placement
-  - Music: royalty-free background bed, low volume under the voiceover</t>
+  - Music: royalty-free background bed, low volume under the voiceover
+  - ---
+  - ## Technical reference (source of truth)
+  - **Screens:** `/sales/my-shift` [M] (Start Shift, stat cards, Shift Summary,
+  - Shift Progress chart, Shift Receipts, Shift Expenses, Past Shift Net Sales
+  - chart, Shift History table, Shift Report preview, Balance Shift, Record
+  - Expense, End Shift) · `/sales/history` (per-shift sales via filters) ·
+  - `/sales/refunds` (per shift)
+  - **User actions (FE hooks):** `useActiveShift` / `useShifts` / `useShiftSales`
+  - (/sales/by-shift) / `useShiftPayments` (/shifts/{id}/payments) /
+  - `useShiftExpenses` (/expenses?shift_id=) · `useClockIn` (start shift) ·
+  - `useClockOut` (end shift + totals: total_sales, total_cash,
+  - total_mobile_money, total_card, counted_cash) · `useUpdateShiftOpeningBalance`
+  - (opening_balance) · `useUpdateShiftBalance` (opening_balance + counted_cash) ·
+  - `useEndShiftAction` (totals math + logout) · `buildShiftCloseReportData` /
+  - `canDownloadShiftClosePdf` / `downloadShiftClosePdf` (report + PDF)
+  - **API endpoints (BE):** `/shifts` CRUD (POST = clock in, PUT = opening balance
+  - / counted cash / clock out + close) · `/shifts/active` (current shift) ·
+  - `/shifts/{id}/payments` (shift payments) · `/sales/by-shift/{id}` (shift
+  - sales) · `/expenses?shift_id={id}` (shift expenses) · `/sales/daily` (day
+  - rollup per shift)</t>
         </is>
       </c>
       <c r="D117" s="5" t="n"/>
@@ -7686,35 +7686,6 @@
 DEMO DATA: A fresh device state with no account.
 CTA: Try free + subscribe
 RELATED: [01-account-auth-security.md](./01-account-auth-security.md)
----
-## Technical reference (source of truth)
-**Screens:** OfflineBanner (amber, dismissible, "you can keep working") ·
-AuthPendingBanner (amber, "your account is pending sync") · SyncProgressBanner
-(progress bar, phase label, per-item count, ETA, pause/failure/success states)
-· SyncHeaderChip in the navbar (spinner + percent) · pending-payment notices in
-Payment history
-**Sync engine (FE):** `syncCoordinator.runSyncCoordinator()` drains the queue in
-ordered tiers (Account, Foundation, Transactions, Closures, Stock), looping
-until empty or offline · `syncEngine.runSyncPipeline()` orders mutations by
-dependency (shift opens -&gt; categories -&gt; roles -&gt; staff -&gt; orders -&gt; sales -&gt;
-sale payments -&gt; refunds -&gt; shift closes -&gt; other updates -&gt; stock adjustments)
-· `mutationQueue` persists queued mutations to IndexedDB + durable localStorage
-backup, with retry counters, stale-syncing recovery (5 min), and per-business
-scoping · offline sales upload in batches of 25 (`SALES_BATCH_SIZE`) with
-retry/backoff, then fall back to per-sale sync; duplicate and ambiguous
-failures are reconciled · offline-created entities get negative local IDs that
-are remapped to server IDs (`entityIdMapper`) · reads use
-`readWithOfflineStrategy()` (server first, client cache/IndexedDB fallback on
-network error, 404, or pre-auth 401) · offline auth: `completeOfflineRegistration`
-(local account + queued `/businesses/register` with maxRetries 10, pendingAuthSync
-flag) and `completeOfflineLogin` (local session token; offline login after
-registering on-device or one online login)
-**API endpoints (BE):** `sync.php` (auth:sanctum + business.active):
-`POST /sync/push` (categories, products, customers, expenses, invoices, sales,
-sale_items, stock_movements, staff_transfers, quick_notes) · `GET /sync/pull?since=`
-· `GET /sync/full` · `sales.php` (auth:sanctum + business.active +
-subscription.active): `POST /sales/batch` (bulk sales sync) · `POST /sales` per
-sale fallback
 PUBLISHED TITLE: Set up Custosell offline. Sign in online later.
 SHORT-FORM VARIANT: Set up Custosell offline. Sign
 PUBLISHED DESCRIPTION: You can create your Custosell account without internet - the registration is saved on the device and synced to the server when you connect. An amber banner shows your account is pending sync, and offline sign-in keeps working after that. Try free + subscribe #custosell #offline #sync #nointernet #Custosell #SmallBusiness
@@ -7724,7 +7695,36 @@
   - Screen-record clips: the Screen flow steps, trimmed to the script beats
   - Captions / subtitles: full on-screen captions exported as a caption file
   - Brand overlay / watermark: Custosell logo, corner placement
-  - Music: royalty-free background bed, low volume under the voiceover</t>
+  - Music: royalty-free background bed, low volume under the voiceover
+  - ---
+  - ## Technical reference (source of truth)
+  - **Screens:** OfflineBanner (amber, dismissible, "you can keep working") ·
+  - AuthPendingBanner (amber, "your account is pending sync") · SyncProgressBanner
+  - (progress bar, phase label, per-item count, ETA, pause/failure/success states)
+  - · SyncHeaderChip in the navbar (spinner + percent) · pending-payment notices in
+  - Payment history
+  - **Sync engine (FE):** `syncCoordinator.runSyncCoordinator()` drains the queue in
+  - ordered tiers (Account, Foundation, Transactions, Closures, Stock), looping
+  - until empty or offline · `syncEngine.runSyncPipeline()` orders mutations by
+  - dependency (shift opens -&gt; categories -&gt; roles -&gt; staff -&gt; orders -&gt; sales -&gt;
+  - sale payments -&gt; refunds -&gt; shift closes -&gt; other updates -&gt; stock adjustments)
+  - · `mutationQueue` persists queued mutations to IndexedDB + durable localStorage
+  - backup, with retry counters, stale-syncing recovery (5 min), and per-business
+  - scoping · offline sales upload in batches of 25 (`SALES_BATCH_SIZE`) with
+  - retry/backoff, then fall back to per-sale sync; duplicate and ambiguous
+  - failures are reconciled · offline-created entities get negative local IDs that
+  - are remapped to server IDs (`entityIdMapper`) · reads use
+  - `readWithOfflineStrategy()` (server first, client cache/IndexedDB fallback on
+  - network error, 404, or pre-auth 401) · offline auth: `completeOfflineRegistration`
+  - (local account + queued `/businesses/register` with maxRetries 10, pendingAuthSync
+  - flag) and `completeOfflineLogin` (local session token; offline login after
+  - registering on-device or one online login)
+  - **API endpoints (BE):** `sync.php` (auth:sanctum + business.active):
+  - `POST /sync/push` (categories, products, customers, expenses, invoices, sales,
+  - sale_items, stock_movements, staff_transfers, quick_notes) · `GET /sync/pull?since=`
+  - · `GET /sync/full` · `sales.php` (auth:sanctum + business.active +
+  - subscription.active): `POST /sales/batch` (bulk sales sync) · `POST /sales` per
+  - sale fallback</t>
         </is>
       </c>
       <c r="D121" s="5" t="n"/>
@@ -8294,35 +8294,6 @@
 DEMO DATA: A device with connectivity toggled off.
 CTA: Try free
 RELATED: [21-offline-sync.md](./21-offline-sync.md)
----
-## Technical reference (source of truth)
-**Screens:** `/expenses/list` [M] (list, filters, CRUD, attachments) ·
-`/expenses/categories` [M] (category manager with per-category budgets) ·
-`/expenses/overview` [M] (stat cards + charts, period/branch filters) ·
-`/expenses/budgets` [M] (personal budgets, shopping lists, PDF download) ·
-`/expenses/income` [M] (income records, personal accounts only)
-**User actions (FE hooks):** `useExpenses` · `useExpense(id)` ·
-`useExpenseSummary` · `useExpenseCategories` · `useCreateExpense` ·
-`useUpdateExpense` · `useDeleteExpense` · `useCreateExpenseCategory` ·
-`useUpdateExpenseCategory` · `useDeleteExpenseCategory` ·
-`useUploadExpenseAttachment` · `useCreateExpenseAttachmentLink` ·
-`useDeleteExpenseAttachment` · `useBudgetsIndex` · `useBudget(id)` ·
-`useCreateBudget` · `useUpdateBudget` · `useDeleteBudget` ·
-`useBudgetDetail` · `useSyncBudgetLines` · `usePurchaseLine` ·
-`useBudgetAffordability` · `useBudgetAlerts` · `useMoneySummary` ·
-`useIncomeSources` · `useCreateIncome` · `useUpdateIncome` ·
-`useDeleteIncome` · `useUploadIncomeAttachment` ·
-`useCreateIncomeAttachmentLink` · `useDeleteIncomeAttachment` ·
-`useIncomeOverview` · `useBudgets` · `downloadBudgetPdf`
-**API endpoints (BE):** `/expenses` (GET/POST + `/expenses/{id}` GET/PUT/PATCH/
-DELETE) · `/expenses/overview` · `/expenses/summary` · `/expenses/budgets` ·
-`/expenses/export` (CSV/XLSX) · `/expenses/by-shift/{shiftId}` ·
-`/expenses/{id}/attachments` (+ `/attachments/link` + `/expense-attachments/{id}`)
-· `/expense-categories` CRUD · `/income-sources` CRUD (+ `/summary` +
-`/income-sources/{id}/attachments` + `/attachments/link` +
-`/income-source-attachments/{id}`) · `/budgets` CRUD (+ `/budgets/{id}/lines`,
-`/lines/{line}/purchase`, `/affordability`, `/download`) · `/money/summary` ·
-`/money/alerts`
 PUBLISHED TITLE: Record expenses even when the internet is gone.
 SHORT-FORM VARIANT: Record expenses even when the internet is gone.
 PUBLISHED DESCRIPTION: Create and edit expenses offline - Custosell saves them instantly with a Pending sync badge (and pending receipt) and syncs automatically when you're back online. Try free #custosell #expenses #budgets #income #Custosell #SmallBusiness
@@ -8332,7 +8303,36 @@
   - Screen-record clips: the Screen flow steps, trimmed to the script beats
   - Captions / subtitles: full on-screen captions exported as a caption file
   - Brand overlay / watermark: Custosell logo, corner placement
-  - Music: royalty-free background bed, low volume under the voiceover</t>
+  - Music: royalty-free background bed, low volume under the voiceover
+  - ---
+  - ## Technical reference (source of truth)
+  - **Screens:** `/expenses/list` [M] (list, filters, CRUD, attachments) ·
+  - `/expenses/categories` [M] (category manager with per-category budgets) ·
+  - `/expenses/overview` [M] (stat cards + charts, period/branch filters) ·
+  - `/expenses/budgets` [M] (personal budgets, shopping lists, PDF download) ·
+  - `/expenses/income` [M] (income records, personal accounts only)
+  - **User actions (FE hooks):** `useExpenses` · `useExpense(id)` ·
+  - `useExpenseSummary` · `useExpenseCategories` · `useCreateExpense` ·
+  - `useUpdateExpense` · `useDeleteExpense` · `useCreateExpenseCategory` ·
+  - `useUpdateExpenseCategory` · `useDeleteExpenseCategory` ·
+  - `useUploadExpenseAttachment` · `useCreateExpenseAttachmentLink` ·
+  - `useDeleteExpenseAttachment` · `useBudgetsIndex` · `useBudget(id)` ·
+  - `useCreateBudget` · `useUpdateBudget` · `useDeleteBudget` ·
+  - `useBudgetDetail` · `useSyncBudgetLines` · `usePurchaseLine` ·
+  - `useBudgetAffordability` · `useBudgetAlerts` · `useMoneySummary` ·
+  - `useIncomeSources` · `useCreateIncome` · `useUpdateIncome` ·
+  - `useDeleteIncome` · `useUploadIncomeAttachment` ·
+  - `useCreateIncomeAttachmentLink` · `useDeleteIncomeAttachment` ·
+  - `useIncomeOverview` · `useBudgets` · `downloadBudgetPdf`
+  - **API endpoints (BE):** `/expenses` (GET/POST + `/expenses/{id}` GET/PUT/PATCH/
+  - DELETE) · `/expenses/overview` · `/expenses/summary` · `/expenses/budgets` ·
+  - `/expenses/export` (CSV/XLSX) · `/expenses/by-shift/{shiftId}` ·
+  - `/expenses/{id}/attachments` (+ `/attachments/link` + `/expense-attachments/{id}`)
+  - · `/expense-categories` CRUD · `/income-sources` CRUD (+ `/summary` +
+  - `/income-sources/{id}/attachments` + `/attachments/link` +
+  - `/income-source-attachments/{id}`) · `/budgets` CRUD (+ `/budgets/{id}/lines`,
+  - `/lines/{line}/purchase`, `/affordability`, `/download`) · `/money/summary` ·
+  - `/money/alerts`</t>
         </is>
       </c>
       <c r="D131" s="5" t="n"/>
@@ -8724,23 +8724,6 @@
 DEMO DATA: A device with connectivity toggled off.
 CTA: Try free
 RELATED: [21-offline-sync.md](./21-offline-sync.md)
----
-## Technical reference (source of truth)
-**Screens:** `/customers` [M] (list, search, add/edit/delete, purchases),
-`/customers/overview` [M] (stats + charts), `/sales/new` billing column
-(checkout picker)
-**User actions (FE hooks):** `useCustomers` · `useCustomer(id)` ·
-`useCustomerOverview` · `useCustomerPurchases(id)` ·
-`useCreateCustomer` · `useUpdateCustomer` · `useDeleteCustomer` ·
-`useResolveCustomerContact` (find-or-create + merge contact) ·
-`useAssignSaleCustomer` (attach customer to an existing sale)
-**API endpoints (BE):** `/customers` (GET/POST) · `/customers/overview` ·
-`/customers/resolve` (find-or-create by id/email/phone, merges contact) ·
-`/customers/{id}` (GET/PUT/PATCH/DELETE) · `/customers/{id}/purchases` ·
-`/sales/{id}/customer` (assign)
-**Overview segments (BE `CustomerService`):** Active (&lt;30 days) · At risk
-(30-90 days) · Lapsed (&gt;90 days) · Never purchased. Frequency buckets: 1 · 2-3 ·
-4-6 · 7+ purchases.
 PUBLISHED TITLE: Add customers even when the internet is gone.
 SHORT-FORM VARIANT: Add customers even when the internet is gone.
 PUBLISHED DESCRIPTION: Create and edit customers while offline - Custosell saves them instantly with a Pending sync badge and syncs automatically when you're back. Try free #custosell #customers #customerlist #purchasehistory #Custosell #SmallBusiness
@@ -8750,7 +8733,24 @@
   - Screen-record clips: the Screen flow steps, trimmed to the script beats
   - Captions / subtitles: full on-screen captions exported as a caption file
   - Brand overlay / watermark: Custosell logo, corner placement
-  - Music: royalty-free background bed, low volume under the voiceover</t>
+  - Music: royalty-free background bed, low volume under the voiceover
+  - ---
+  - ## Technical reference (source of truth)
+  - **Screens:** `/customers` [M] (list, search, add/edit/delete, purchases),
+  - `/customers/overview` [M] (stats + charts), `/sales/new` billing column
+  - (checkout picker)
+  - **User actions (FE hooks):** `useCustomers` · `useCustomer(id)` ·
+  - `useCustomerOverview` · `useCustomerPurchases(id)` ·
+  - `useCreateCustomer` · `useUpdateCustomer` · `useDeleteCustomer` ·
+  - `useResolveCustomerContact` (find-or-create + merge contact) ·
+  - `useAssignSaleCustomer` (attach customer to an existing sale)
+  - **API endpoints (BE):** `/customers` (GET/POST) · `/customers/overview` ·
+  - `/customers/resolve` (find-or-create by id/email/phone, merges contact) ·
+  - `/customers/{id}` (GET/PUT/PATCH/DELETE) · `/customers/{id}/purchases` ·
+  - `/sales/{id}/customer` (assign)
+  - **Overview segments (BE `CustomerService`):** Active (&lt;30 days) · At risk
+  - (30-90 days) · Lapsed (&gt;90 days) · Never purchased. Frequency buckets: 1 · 2-3 ·
+  - 4-6 · 7+ purchases.</t>
         </is>
       </c>
       <c r="D138" s="5" t="n"/>
@@ -9750,7 +9750,7 @@
     <row r="156">
       <c r="A156" s="5" t="inlineStr">
         <is>
-          <t>MKT-18 List products on your public shop</t>
+          <t>MKT-18 Put your catalog in front of customers</t>
         </is>
       </c>
       <c r="B156" s="5" t="inlineStr">
@@ -9839,26 +9839,6 @@
 DEMO DATA: A device with connectivity toggled off.
 CTA: Try free
 RELATED: [21-offline-sync.md](./21-offline-sync.md)
----
-## Technical reference (source of truth)
-**Screens:** `/inventory/marketplace` [M], `/inventory/purchase-orders` [M],
-`/inventory/incoming-orders` [M]
-**User actions (FE hooks):** `useMarketplaceBusinesses` ·
-`useMarketplaceProducts` · `useMySuppliers` · `useAddSupplier` ·
-`useRemoveSupplier` · `useCreatePurchaseOrder` · `useUpdatePurchaseOrder` ·
-`useSubmitPurchaseOrder` · `useCancelPurchaseOrder` ·
-`useDeletePurchaseOrder` · `useAcceptPurchaseOrder` ·
-`useRejectPurchaseOrder` · `useFulfillPurchaseOrder` ·
-`useReceivePurchaseOrder` · `usePurchaseOrders` ·
-`useIncomingPurchaseOrders` · `usePurchaseOrder` ·
-`useUpdateSupplyListing` · `useUpdateStorefrontListing`
-**API endpoints (BE):** `/marketplace/businesses` ·
-`/marketplace/businesses/{id}/products` · `/marketplace/suppliers`
-(GET/POST) + `/marketplace/suppliers/{sellerBusinessId}` (DELETE) ·
-`/purchase-orders` (GET/POST) + `/purchase-orders/{id}`
-(GET/PUT/DELETE) + `/purchase-orders/{id}/submit|cancel|accept|reject|
-fulfill|receive` · `/purchase-orders/incoming` ·
-`/products/{id}/supply-listing` · `/products/{id}/storefront-listing`
 PUBLISHED TITLE: Know exactly what needs a connection.
 SHORT-FORM VARIANT: Know exactly what needs a connection.
 PUBLISHED DESCRIPTION: Marketplace browsing, ordering, and order management need the internet - see how Custosell tells you clearly and keeps your local work safe. Try free #custosell #marketplace #purchaseorder #suppliers #Custosell #SmallBusiness
@@ -9868,7 +9848,27 @@
   - Screen-record clips: the Screen flow steps, trimmed to the script beats
   - Captions / subtitles: full on-screen captions exported as a caption file
   - Brand overlay / watermark: Custosell logo, corner placement
-  - Music: royalty-free background bed, low volume under the voiceover</t>
+  - Music: royalty-free background bed, low volume under the voiceover
+  - ---
+  - ## Technical reference (source of truth)
+  - **Screens:** `/inventory/marketplace` [M], `/inventory/purchase-orders` [M],
+  - `/inventory/incoming-orders` [M]
+  - **User actions (FE hooks):** `useMarketplaceBusinesses` ·
+  - `useMarketplaceProducts` · `useMySuppliers` · `useAddSupplier` ·
+  - `useRemoveSupplier` · `useCreatePurchaseOrder` · `useUpdatePurchaseOrder` ·
+  - `useSubmitPurchaseOrder` · `useCancelPurchaseOrder` ·
+  - `useDeletePurchaseOrder` · `useAcceptPurchaseOrder` ·
+  - `useRejectPurchaseOrder` · `useFulfillPurchaseOrder` ·
+  - `useReceivePurchaseOrder` · `usePurchaseOrders` ·
+  - `useIncomingPurchaseOrders` · `usePurchaseOrder` ·
+  - `useUpdateSupplyListing` · `useUpdateStorefrontListing`
+  - **API endpoints (BE):** `/marketplace/businesses` ·
+  - `/marketplace/businesses/{id}/products` · `/marketplace/suppliers`
+  - (GET/POST) + `/marketplace/suppliers/{sellerBusinessId}` (DELETE) ·
+  - `/purchase-orders` (GET/POST) + `/purchase-orders/{id}`
+  - (GET/PUT/DELETE) + `/purchase-orders/{id}/submit|cancel|accept|reject|
+  - fulfill|receive` · `/purchase-orders/incoming` ·
+  - `/products/{id}/supply-listing` · `/products/{id}/storefront-listing`</t>
         </is>
       </c>
       <c r="D157" s="5" t="n"/>
@@ -11399,37 +11399,6 @@
 DEMO DATA: A project and a few staff accounts.
 CTA: Try free
 RELATED: [17-settings.md](./17-settings.md)
----
-## Technical reference (source of truth)
-**Screens:** `/estimates` [M] (list + stat cards + New estimate drawer) ·
-`/estimates/{id}` [M] (detail: send/email/approve/reject/convert/PDF/duplicate +
-line items, versions, notes) · `/estimates/templates` [M] (template cards) ·
-`/estimates/insights` [M] (win rate, margin, trends) ·
-`/estimates/projects` [M] (project list with budget vs actual) ·
-`/estimates/projects/{id}` [M] (overview/tasks/timesheets/board/documents/
-allocations) · `/estimates/boards` [M] (estimates-workspace kanban boards -
-"My boards" personal + "Project boards", New personal board drawer)
-**User actions (FE hooks):** `useEstimates` · `useEstimate` ·
-`useCreateEstimate` · `useUpdateEstimate` · `useDeleteEstimate` ·
-`useSendEstimate` (status only) · `useEmailEstimate` (real email) ·
-`useApproveEstimate` · `useRejectEstimate` · `useDuplicateEstimate` ·
-`useEstimateVersions` · `useConvertEstimateToInvoice` ·
-`useConvertEstimateToProject` · `useEstimateAnalytics` · `useEstimateTemplates`
-(+ CRUD) · `useProjects` · `useProject` · `useCreateProject` ·
-`useUpdateProject` · `useDeleteProject` · `useMyProjects` ·
-`useCreateProjectTask`/`useUpdateProjectTask`/`useDeleteProjectTask` ·
-`useCreateTimesheetEntry`/`useDeleteTimesheetEntry` ·
-`useCreateCostAllocation`/`useDeleteCostAllocation` · `useProjectBudgetSummary`
-· `useProjectProfitability` · `useProjectBoard` · `useProjectBoardKanban` ·
-`useProjectMembers`/`useAddProjectMember`/`useUpdateProjectMember`/
-`useRemoveProjectMember` · `viewEstimatePdf`/`downloadEstimatePdf` ·
-`usePipelineBoards` (estimatesWorkspace: true) · `useCreatePipelineBoard`
-(personal boards, workspace=estimates, private by default) ·
-`usePipelineKanban` · `filterBoardsForWorkspace`/`boardBelongsToEstimatesWorkspace`/
-`boardUsesTaskTerminology` (task/card language for project + estimates boards) ·
-`useProjectBoard`/`useProjectBoardKanban` (project board via project id) ·
-`isLimitedEstimatesUser`/`getEstimatesModuleDefaultRoute` (board-only users
-land on `/estimates/boards`)
 PUBLISHED TITLE: Right people, right access, one project.
 SHORT-FORM VARIANT: Right people
 PUBLISHED DESCRIPTION: Invite staff to a project as Viewer, Contributor, or Manager, control who edits and who manages the team, and keep the owner locked in. Try free #custosell #estimates #projects #templates #Custosell #SmallBusiness
@@ -11439,7 +11408,38 @@
   - Screen-record clips: the Screen flow steps, trimmed to the script beats
   - Captions / subtitles: full on-screen captions exported as a caption file
   - Brand overlay / watermark: Custosell logo, corner placement
-  - Music: royalty-free background bed, low volume under the voiceover</t>
+  - Music: royalty-free background bed, low volume under the voiceover
+  - ---
+  - ## Technical reference (source of truth)
+  - **Screens:** `/estimates` [M] (list + stat cards + New estimate drawer) ·
+  - `/estimates/{id}` [M] (detail: send/email/approve/reject/convert/PDF/duplicate +
+  - line items, versions, notes) · `/estimates/templates` [M] (template cards) ·
+  - `/estimates/insights` [M] (win rate, margin, trends) ·
+  - `/estimates/projects` [M] (project list with budget vs actual) ·
+  - `/estimates/projects/{id}` [M] (overview/tasks/timesheets/board/documents/
+  - allocations) · `/estimates/boards` [M] (estimates-workspace kanban boards -
+  - "My boards" personal + "Project boards", New personal board drawer)
+  - **User actions (FE hooks):** `useEstimates` · `useEstimate` ·
+  - `useCreateEstimate` · `useUpdateEstimate` · `useDeleteEstimate` ·
+  - `useSendEstimate` (status only) · `useEmailEstimate` (real email) ·
+  - `useApproveEstimate` · `useRejectEstimate` · `useDuplicateEstimate` ·
+  - `useEstimateVersions` · `useConvertEstimateToInvoice` ·
+  - `useConvertEstimateToProject` · `useEstimateAnalytics` · `useEstimateTemplates`
+  - (+ CRUD) · `useProjects` · `useProject` · `useCreateProject` ·
+  - `useUpdateProject` · `useDeleteProject` · `useMyProjects` ·
+  - `useCreateProjectTask`/`useUpdateProjectTask`/`useDeleteProjectTask` ·
+  - `useCreateTimesheetEntry`/`useDeleteTimesheetEntry` ·
+  - `useCreateCostAllocation`/`useDeleteCostAllocation` · `useProjectBudgetSummary`
+  - · `useProjectProfitability` · `useProjectBoard` · `useProjectBoardKanban` ·
+  - `useProjectMembers`/`useAddProjectMember`/`useUpdateProjectMember`/
+  - `useRemoveProjectMember` · `viewEstimatePdf`/`downloadEstimatePdf` ·
+  - `usePipelineBoards` (estimatesWorkspace: true) · `useCreatePipelineBoard`
+  - (personal boards, workspace=estimates, private by default) ·
+  - `usePipelineKanban` · `filterBoardsForWorkspace`/`boardBelongsToEstimatesWorkspace`/
+  - `boardUsesTaskTerminology` (task/card language for project + estimates boards) ·
+  - `useProjectBoard`/`useProjectBoardKanban` (project board via project id) ·
+  - `isLimitedEstimatesUser`/`getEstimatesModuleDefaultRoute` (board-only users
+  - land on `/estimates/boards`)</t>
         </is>
       </c>
       <c r="D183" s="5" t="n"/>
@@ -11551,7 +11551,7 @@
 RELATED: [02-dashboard-reports.md](./02-dashboard-reports.md)
 PUBLISHED TITLE: Chart of accounts, explained for shop owners.
 SHORT-FORM VARIANT: Chart of accounts
-PUBLISHED DESCRIPTION: A plain-English tour of the chart of accounts on Custosell - assets, liabilities, equity, revenue, expenses - in flat view or as a parent- child tree, and how each account feeds your reports. Try free + subscribe #custosell #accounting #bookkeeping #journal #Custosell #SmallBusiness
+PUBLISHED DESCRIPTION: A plain-English tour of the chart of accounts on Custosell - assets, liabilities, equity, revenue, expenses - in flat view or as a parent-child tree, and how each account feeds your reports. Try free + subscribe #custosell #accounting #bookkeeping #journal #Custosell #SmallBusiness
 TAGS: custosell, accounting, bookkeeping, journal, trial balance, income statement, balance sheet, vat, how to, tutorial, walkthrough, tips
 VIDEO ASSETS:
   - Thumbnail: bold text "Assets. Revenue. Expenses. It's that simple." over a bright screenshot of the action
@@ -12196,38 +12196,6 @@
 DEMO DATA: A small Excel file with accounts or entries.
 CTA: Try free
 RELATED: [17-settings.md](./17-settings.md)
----
-## Technical reference (source of truth)
-**Screens:** `/accounting/statements` [M] (5 report cards + PDF export) ·
-`/accounting/chart-of-accounts` [M] (flat/tree, add, import/export) ·
-`/accounting/journal-entries` [M] (list, new entry, post/reverse, import/export)
-· `/accounting/trial-balance` [M] · `/accounting/income-statement` [M] ·
-`/accounting/balance-sheet` [M] · `/accounting/ratios` [M] (trends + download)
-· `/accounting/periods` [M] (close/reopen) · `/accounting/fixed-assets` [M]
-(register, run depreciation, schedule) · `/accounting/settings` [M] (seed COA,
-inventory reconciliation)
-**User actions (FE hooks):** `useChartOfAccounts` · `useChartOfAccountsTree` ·
-`useCreateChartOfAccount` · `useUpdateChartOfAccount` ·
-`useDeleteChartOfAccount` · `useAccountingPeriods` · `useCurrentPeriod` ·
-`useClosePeriod` · `useJournalEntries` · `useJournalEntry` ·
-`useCreateJournalEntry` · `usePostJournalEntry` · `useReverseJournalEntry` ·
-`useDeleteJournalEntry` · `useTrialBalance` · `useIncomeStatement` ·
-`useBalanceSheet` · `useCashFlow` · `useEquity` · `useRatios` ·
-`useRatioTrends` · `useFixedAssets` · `useFixedAsset` · `useCreateFixedAsset` ·
-`useUpdateFixedAsset` · `useRunDepreciation` · `useFixedAssetSchedule` ·
-`useInventoryReconciliation` · `usePostOpeningInventory`
-**API endpoints (BE):** `/chart-of-accounts` CRUD + `/tree` + `/import-template`
-+ `/import` + `/export` · `/accounting-periods` + `/current` + `/{id}/close` +
-`/{id}/reopen` · `/journal-entries` CRUD + `/import-template` + `/import` +
-`/export` + `/{id}/lines` + `/{id}/post` + `/{id}/reverse` ·
-`/general-ledger` + `/trial-balance` + `/profit-loss` + `/balance-sheet` +
-`/cash-flow` + `/equity` · `/fixed-assets` CRUD + `/run-depreciation` +
-`/{id}/schedule` · `/ratios` + `/ratios/trends` · `/inventory/reconciliation` +
-`/inventory/opening-balance` · `/accounting/export/{type}` (PDF/XLSX)
-**Auto-journaling events (BE):** `SaleCreatedForAccounting` ·
-`SaleRefundedForAccounting` · `ExpenseCreatedForAccounting` ·
-`InvoiceSentForAccounting` · `InvoicePaidForAccounting` ·
-`PaymentRecordedForAccounting` · `PayoutCompletedForAccounting`
 PUBLISHED TITLE: Move your books in and out - cleanly.
 SHORT-FORM VARIANT: Move your books in and out
 PUBLISHED DESCRIPTION: Download a template, import your chart of accounts or journal entries from Excel/CSV, and export current data - with per-row validation so you always know what landed. Try free #custosell #accounting #bookkeeping #journal #Custosell #SmallBusiness
@@ -12237,7 +12205,39 @@
   - Screen-record clips: the Screen flow steps, trimmed to the script beats
   - Captions / subtitles: full on-screen captions exported as a caption file
   - Brand overlay / watermark: Custosell logo, corner placement
-  - Music: royalty-free background bed, low volume under the voiceover</t>
+  - Music: royalty-free background bed, low volume under the voiceover
+  - ---
+  - ## Technical reference (source of truth)
+  - **Screens:** `/accounting/statements` [M] (5 report cards + PDF export) ·
+  - `/accounting/chart-of-accounts` [M] (flat/tree, add, import/export) ·
+  - `/accounting/journal-entries` [M] (list, new entry, post/reverse, import/export)
+  - · `/accounting/trial-balance` [M] · `/accounting/income-statement` [M] ·
+  - `/accounting/balance-sheet` [M] · `/accounting/ratios` [M] (trends + download)
+  - · `/accounting/periods` [M] (close/reopen) · `/accounting/fixed-assets` [M]
+  - (register, run depreciation, schedule) · `/accounting/settings` [M] (seed COA,
+  - inventory reconciliation)
+  - **User actions (FE hooks):** `useChartOfAccounts` · `useChartOfAccountsTree` ·
+  - `useCreateChartOfAccount` · `useUpdateChartOfAccount` ·
+  - `useDeleteChartOfAccount` · `useAccountingPeriods` · `useCurrentPeriod` ·
+  - `useClosePeriod` · `useJournalEntries` · `useJournalEntry` ·
+  - `useCreateJournalEntry` · `usePostJournalEntry` · `useReverseJournalEntry` ·
+  - `useDeleteJournalEntry` · `useTrialBalance` · `useIncomeStatement` ·
+  - `useBalanceSheet` · `useCashFlow` · `useEquity` · `useRatios` ·
+  - `useRatioTrends` · `useFixedAssets` · `useFixedAsset` · `useCreateFixedAsset` ·
+  - `useUpdateFixedAsset` · `useRunDepreciation` · `useFixedAssetSchedule` ·
+  - `useInventoryReconciliation` · `usePostOpeningInventory`
+  - **API endpoints (BE):** `/chart-of-accounts` CRUD + `/tree` + `/import-template`
+  - + `/import` + `/export` · `/accounting-periods` + `/current` + `/{id}/close` +
+  - `/{id}/reopen` · `/journal-entries` CRUD + `/import-template` + `/import` +
+  - `/export` + `/{id}/lines` + `/{id}/post` + `/{id}/reverse` ·
+  - `/general-ledger` + `/trial-balance` + `/profit-loss` + `/balance-sheet` +
+  - `/cash-flow` + `/equity` · `/fixed-assets` CRUD + `/run-depreciation` +
+  - `/{id}/schedule` · `/ratios` + `/ratios/trends` · `/inventory/reconciliation` +
+  - `/inventory/opening-balance` · `/accounting/export/{type}` (PDF/XLSX)
+  - **Auto-journaling events (BE):** `SaleCreatedForAccounting` ·
+  - `SaleRefundedForAccounting` · `ExpenseCreatedForAccounting` ·
+  - `InvoiceSentForAccounting` · `InvoicePaidForAccounting` ·
+  - `PaymentRecordedForAccounting` · `PayoutCompletedForAccounting`</t>
         </is>
       </c>
       <c r="D196" s="5" t="n"/>
@@ -12804,33 +12804,6 @@
 DEMO DATA: A few staff members actively filing documents.
 CTA: Try free
 RELATED: [17-settings.md](./17-settings.md)
----
-## Technical reference (source of truth)
-**Screens:** `/documents` [M] (cabinet cards + search + New cabinet) ·
-`/documents/cabinets/{id}` [M] (explorer: folder tree, upload/link/import,
-access, preview/edit, email, export, activity)
-**User actions (FE hooks):** `useDocumentCabinets` · `useDocumentCabinet` ·
-`useCreateDocumentCabinet` · `useUpdateDocumentCabinet` ·
-`useDeleteDocumentCabinet` · `useDocumentFolderTree` ·
-`useDocumentFolderChildren` · `useDocumentFolderContents` ·
-`useCreateDocumentFolder` · `useUpdateDocumentFolder` ·
-`useDeleteDocumentFolder` · `useDocuments` (infinite list) · `useDocument` ·
-`useUploadDocument` · `useCreateDocumentLink` · `useUpdateDocument` ·
-`useDeleteDocument` · `useDocumentContent` · `useUpdateDocumentContent` ·
-`useRecordDocumentView` · `useRecordDocumentDownload` ·
-`useDocumentAccessibleMembers` · `useDocumentActivity` · `useDocumentTags` ·
-`useDocumentsVaultAppearance` · `useUpdateDocumentsVaultAppearance`
-**API endpoints (BE):** `/documents` GET + `/documents/upload` +
-`/documents/link` + `/documents/{id}` GET/PATCH/DELETE + `/{id}/view` +
-`/{id}/download` + `/{id}/email` + `/{id}/content` GET/PUT ·
-`/documents/cabinets` CRUD + `/documents/activity` + `/documents/vault-appearance`
-GET/PATCH + `/documents/accessible-members` + `/documents/tags` GET/POST ·
-`/documents/folders/tree` + `/documents/folders/children` + `/documents/folders`
-POST + `/documents/folders/{id}` GET/PATCH/DELETE + `/{id}/contents` +
-`/{id}/export` (zip) + `/{id}/email`
-**Vault client helpers (FE):** `uploadDocumentWithProgress` ·
-`downloadFileWithProgress` · `downloadFolderExportWithProgress` ·
-`importFolderTree` (recreates a local folder tree in the vault)
 PUBLISHED TITLE: Every upload, move, and email - on record.
 SHORT-FORM VARIANT: Every upload, move, and email
 PUBLISHED DESCRIPTION: Open the vault activity feed to see who uploaded, moved, renamed, emailed, or deleted what - a full audit trail for your documents. Try free #custosell #documents #filestorage #vault #Custosell #SmallBusiness
@@ -12840,7 +12813,34 @@
   - Screen-record clips: the Screen flow steps, trimmed to the script beats
   - Captions / subtitles: full on-screen captions exported as a caption file
   - Brand overlay / watermark: Custosell logo, corner placement
-  - Music: royalty-free background bed, low volume under the voiceover</t>
+  - Music: royalty-free background bed, low volume under the voiceover
+  - ---
+  - ## Technical reference (source of truth)
+  - **Screens:** `/documents` [M] (cabinet cards + search + New cabinet) ·
+  - `/documents/cabinets/{id}` [M] (explorer: folder tree, upload/link/import,
+  - access, preview/edit, email, export, activity)
+  - **User actions (FE hooks):** `useDocumentCabinets` · `useDocumentCabinet` ·
+  - `useCreateDocumentCabinet` · `useUpdateDocumentCabinet` ·
+  - `useDeleteDocumentCabinet` · `useDocumentFolderTree` ·
+  - `useDocumentFolderChildren` · `useDocumentFolderContents` ·
+  - `useCreateDocumentFolder` · `useUpdateDocumentFolder` ·
+  - `useDeleteDocumentFolder` · `useDocuments` (infinite list) · `useDocument` ·
+  - `useUploadDocument` · `useCreateDocumentLink` · `useUpdateDocument` ·
+  - `useDeleteDocument` · `useDocumentContent` · `useUpdateDocumentContent` ·
+  - `useRecordDocumentView` · `useRecordDocumentDownload` ·
+  - `useDocumentAccessibleMembers` · `useDocumentActivity` · `useDocumentTags` ·
+  - `useDocumentsVaultAppearance` · `useUpdateDocumentsVaultAppearance`
+  - **API endpoints (BE):** `/documents` GET + `/documents/upload` +
+  - `/documents/link` + `/documents/{id}` GET/PATCH/DELETE + `/{id}/view` +
+  - `/{id}/download` + `/{id}/email` + `/{id}/content` GET/PUT ·
+  - `/documents/cabinets` CRUD + `/documents/activity` + `/documents/vault-appearance`
+  - GET/PATCH + `/documents/accessible-members` + `/documents/tags` GET/POST ·
+  - `/documents/folders/tree` + `/documents/folders/children` + `/documents/folders`
+  - POST + `/documents/folders/{id}` GET/PATCH/DELETE + `/{id}/contents` +
+  - `/{id}/export` (zip) + `/{id}/email`
+  - **Vault client helpers (FE):** `uploadDocumentWithProgress` ·
+  - `downloadFileWithProgress` · `downloadFolderExportWithProgress` ·
+  - `importFolderTree` (recreates a local folder tree in the vault)</t>
         </is>
       </c>
       <c r="D206" s="5" t="n"/>
@@ -13177,7 +13177,7 @@
 CTA: Try free
 RELATED: [19-notifications-webpush.md](./19-notifications-webpush.md)
 PUBLISHED TITLE: The fortune is in the follow-up.
-SHORT-FORM VARIANT: The fortune is
+SHORT-FORM VARIANT: The follow-up is the fortune
 PUBLISHED DESCRIPTION: Set a reminder on any lead - when and how (in-app, email, or both) - and Custosell nags you so no deal goes cold. Try free #custosell #crm #pipeline #leads #Custosell #SmallBusiness
 TAGS: custosell, crm, pipeline, leads, sales funnel, kanban, deals, how to, tutorial, walkthrough, tips
 VIDEO ASSETS:
@@ -13867,59 +13867,6 @@
 DEMO DATA: A recently won deal.
 CTA: Try free
 RELATED: [11-pipeline-crm.md](./11-pipeline-crm.md)
----
-## Technical reference (source of truth)
-**Screens:** `/pipeline/boards` [M] (board directory + search) ·
-`/pipeline/boards/{boardRef}` [M] (full-screen kanban/calendar/members/progress/
-fame + conversation + collaboration) · `/pipeline/my-work` [M] (my open leads) ·
-`/pipeline/leads` [M] (all leads with filters) · `/pipeline/insights` [M] ·
-`/pipeline/settings` [M] (sources, labels, custom fields, boards directory) ·
-`/pipeline/referrals` · `/book/{token}` + `/book/{token}/check/{reference}`
-[public]
-**User actions (FE hooks):** `usePipelineBoards` · `usePipelineBoard` ·
-`usePipelineKanban` · `useCreatePipelineBoard` · `useUpdatePipelineBoard` ·
-`useDuplicatePipelineBoard` · `useDeletePipelineBoard` ·
-`useCreatePipelineStage` · `useUpdatePipelineStage` · `useDeletePipelineStage`
-· `useReorderPipelineStages` · `usePipelineLeads` · `usePipelineLead` ·
-`useCreatePipelineLead` · `useUpdatePipelineLead` · `useMovePipelineLead` ·
-`useConvertPipelineLead` · `useDeletePipelineLead` · `usePipelineSources`
-(+ CRUD) · `usePipelineLabels` (+ CRUD) · `useCreatePipelineChecklist` +
-items (+ update/delete) · `useAddPipelineActivity`/`useUpdatePipelineActivity`/
-`useDeletePipelineActivity` · `useToggleActivityReaction` ·
-`useLeadReminders`/`useCreateLeadReminder`/`useCancelLeadReminder` ·
-`useBoardAnnouncements`/`useCreateBoardAnnouncement`/`useSetAnnouncementRead` ·
-`useBoardPolls`/`useCreateBoardPoll`/`useVotePoll`/`useRemovePollVote` ·
-`useBoardConversationSummary`/`useBoardConversationMessages`/`usePostBoardMessage`
-(+ update/delete/react/pin/read) · `useBoardAutomations`/`useSyncBoardAutomations`
-· `useBoardResources`(+ CRUD + members) · `useBoardTemplates`/`useApplyBoardTemplate`
-· `usePipelineCalendar`/`useAllBoardsCalendar` · `usePipelineInsights` ·
-`useBoardProgressSummary`/`useMyBoardProgress`/`useBoardTargets`/
-`useCreateBoardTarget`/`useUpdateBoardTarget`/`useArchiveBoardTarget`/
-`useDecomposeTargetPreview`/`useExportBoardProgress` · `useWallFamePosts`(+ CRUD)
-· `useBookingInfo`/`useBookingSlots`/`useCreateBooking`/`useCheckBooking`/
-`useBookingSettings`(+ update/regenerate token)/`useApproveBooking`/
-`useCompleteBooking`/`useRejectBooking`/`useClearBooking` ·
-`useScheduleMeeting`/`useCreateMeeting`/`useUpdateMeeting`/`useDeleteMeeting` ·
-`usePipelineMemberRoster`
-**API endpoints (BE):** `/pipeline/boards` CRUD + `/kanban` + `/calendar` +
-`/duplicate` + `/background` + `/import-template` + `/import` +
-`/team-members` · `/pipeline/boards/{id}/stages` + `/stages/reorder` +
-`/pipeline/stages/{id}` · `/pipeline/leads` CRUD + `/{id}/stage` +
-`/{id}/convert` + `/{id}/activities` + `/{id}/attachments` (+ `/link`) +
-`/{id}/checklists` + items + `/{id}/meta-values` + `/{id}/links` +
-`/{id}/reminders` · `/pipeline/sources` CRUD · `/pipeline/labels` CRUD ·
-`/pipeline/insights` · `/pipeline/boards/{id}/collaboration-summary` +
-`/announcements` + `/polls` (+ vote) + `/conversation/*` + `/automations` +
-`/resources` (+ upload/link/view/download) + `/progress/summary` + `/progress/my`
-+ `/progress/config` + `/progress/export` + `/targets` (+ decompose-preview) ·
-`/pipeline/board-templates` + `/apply-template` · `/pipeline/wall-of-fame` CRUD
-· `/pipeline/boards/{id}/booking-settings` (+ regenerate-token) +
-`/pipeline/leads/{id}/approve-booking|complete-booking|reject-booking|
-clear-booking|schedule-meeting` + `/pipeline/meetings/{id}` ·
-`/public/book/{token}` + `/slots` + `/check/{reference}`
-**Route middleware (BE):** `auth:sanctum` · `business.active` ·
-`subscription.active` · `pipeline.access` (EnsurePipelineModuleAccess) - public
-booking routes unauthenticated
 PUBLISHED TITLE: Closed it? Put it on the wall.
 SHORT-FORM VARIANT: Closed it? Put it on the wall.
 PUBLISHED DESCRIPTION: Post quotes, shoutouts, performers, and milestones to the board's wall of fame - a fun, motivating feed your team sees when they open the board. Try free #custosell #crm #pipeline #leads #Custosell #SmallBusiness
@@ -13929,7 +13876,60 @@
   - Screen-record clips: the Screen flow steps, trimmed to the script beats
   - Captions / subtitles: full on-screen captions exported as a caption file
   - Brand overlay / watermark: Custosell logo, corner placement
-  - Music: royalty-free background bed, low volume under the voiceover</t>
+  - Music: royalty-free background bed, low volume under the voiceover
+  - ---
+  - ## Technical reference (source of truth)
+  - **Screens:** `/pipeline/boards` [M] (board directory + search) ·
+  - `/pipeline/boards/{boardRef}` [M] (full-screen kanban/calendar/members/progress/
+  - fame + conversation + collaboration) · `/pipeline/my-work` [M] (my open leads) ·
+  - `/pipeline/leads` [M] (all leads with filters) · `/pipeline/insights` [M] ·
+  - `/pipeline/settings` [M] (sources, labels, custom fields, boards directory) ·
+  - `/pipeline/referrals` · `/book/{token}` + `/book/{token}/check/{reference}`
+  - [public]
+  - **User actions (FE hooks):** `usePipelineBoards` · `usePipelineBoard` ·
+  - `usePipelineKanban` · `useCreatePipelineBoard` · `useUpdatePipelineBoard` ·
+  - `useDuplicatePipelineBoard` · `useDeletePipelineBoard` ·
+  - `useCreatePipelineStage` · `useUpdatePipelineStage` · `useDeletePipelineStage`
+  - · `useReorderPipelineStages` · `usePipelineLeads` · `usePipelineLead` ·
+  - `useCreatePipelineLead` · `useUpdatePipelineLead` · `useMovePipelineLead` ·
+  - `useConvertPipelineLead` · `useDeletePipelineLead` · `usePipelineSources`
+  - (+ CRUD) · `usePipelineLabels` (+ CRUD) · `useCreatePipelineChecklist` +
+  - items (+ update/delete) · `useAddPipelineActivity`/`useUpdatePipelineActivity`/
+  - `useDeletePipelineActivity` · `useToggleActivityReaction` ·
+  - `useLeadReminders`/`useCreateLeadReminder`/`useCancelLeadReminder` ·
+  - `useBoardAnnouncements`/`useCreateBoardAnnouncement`/`useSetAnnouncementRead` ·
+  - `useBoardPolls`/`useCreateBoardPoll`/`useVotePoll`/`useRemovePollVote` ·
+  - `useBoardConversationSummary`/`useBoardConversationMessages`/`usePostBoardMessage`
+  - (+ update/delete/react/pin/read) · `useBoardAutomations`/`useSyncBoardAutomations`
+  - · `useBoardResources`(+ CRUD + members) · `useBoardTemplates`/`useApplyBoardTemplate`
+  - · `usePipelineCalendar`/`useAllBoardsCalendar` · `usePipelineInsights` ·
+  - `useBoardProgressSummary`/`useMyBoardProgress`/`useBoardTargets`/
+  - `useCreateBoardTarget`/`useUpdateBoardTarget`/`useArchiveBoardTarget`/
+  - `useDecomposeTargetPreview`/`useExportBoardProgress` · `useWallFamePosts`(+ CRUD)
+  - · `useBookingInfo`/`useBookingSlots`/`useCreateBooking`/`useCheckBooking`/
+  - `useBookingSettings`(+ update/regenerate token)/`useApproveBooking`/
+  - `useCompleteBooking`/`useRejectBooking`/`useClearBooking` ·
+  - `useScheduleMeeting`/`useCreateMeeting`/`useUpdateMeeting`/`useDeleteMeeting` ·
+  - `usePipelineMemberRoster`
+  - **API endpoints (BE):** `/pipeline/boards` CRUD + `/kanban` + `/calendar` +
+  - `/duplicate` + `/background` + `/import-template` + `/import` +
+  - `/team-members` · `/pipeline/boards/{id}/stages` + `/stages/reorder` +
+  - `/pipeline/stages/{id}` · `/pipeline/leads` CRUD + `/{id}/stage` +
+  - `/{id}/convert` + `/{id}/activities` + `/{id}/attachments` (+ `/link`) +
+  - `/{id}/checklists` + items + `/{id}/meta-values` + `/{id}/links` +
+  - `/{id}/reminders` · `/pipeline/sources` CRUD · `/pipeline/labels` CRUD ·
+  - `/pipeline/insights` · `/pipeline/boards/{id}/collaboration-summary` +
+  - `/announcements` + `/polls` (+ vote) + `/conversation/*` + `/automations` +
+  - `/resources` (+ upload/link/view/download) + `/progress/summary` + `/progress/my`
+  - + `/progress/config` + `/progress/export` + `/targets` (+ decompose-preview) ·
+  - `/pipeline/board-templates` + `/apply-template` · `/pipeline/wall-of-fame` CRUD
+  - · `/pipeline/boards/{id}/booking-settings` (+ regenerate-token) +
+  - `/pipeline/leads/{id}/approve-booking|complete-booking|reject-booking|
+  - clear-booking|schedule-meeting` + `/pipeline/meetings/{id}` ·
+  - `/public/book/{token}` + `/slots` + `/check/{reference}`
+  - **Route middleware (BE):** `auth:sanctum` · `business.active` ·
+  - `subscription.active` · `pipeline.access` (EnsurePipelineModuleAccess) - public
+  - booking routes unauthenticated</t>
         </is>
       </c>
       <c r="D224" s="5" t="n"/>
@@ -14623,65 +14623,6 @@
 DEMO DATA: A published shop and social link URLs.
 CTA: Try free
 RELATED: [17-settings.md](./17-settings.md)
----
-## Technical reference (source of truth)
-**Screens (buyer):** `/discover` [M] (Businesses / Products tabs, infinite
-catalogs) · `/discover/shop/{slug}` [M] (shop catalog, filters, product modal,
-QR, social) · `/discover/my-orders` [M] (status tabs, cancel/delete, receipt,
-invoice) · `/discover/wishlist` [M] · `/discover/favorites` [M] · `/{@slug}`
-and `/{@slug}/p/{productSlug}` [M] (public share handles that redirect into the
-app). Seller setup lives in Settings -&gt; Sales channels (`BusinessStorefrontCard`,
-`ShopUsernameField`, QR download) and Inventory -&gt; products
-(`ProductStorefrontListingSection`, bulk list/unlist, image upload).
-**User actions (FE hooks):** Catalog: `useStorefrontShopsInfinite` ·
-`useStorefrontDiscoverInfinite` · `useStorefrontFacets` ·
-`useStorefrontCategories` · `useStorefrontShop` ·
-`useStorefrontShopProductsInfinite` · `useStorefrontShopProduct`. Orders:
-`useMyStorefrontOrdersList` (30s poll) · `useMyStorefrontOrdersCount` ·
-`usePlaceStorefrontOrder` · `useCancelMyStorefrontOrder` ·
-`useDeleteMyStorefrontOrder` · `fetchMyStorefrontOrderSale` ·
-`fetchMyStorefrontOrderInvoice`. Wishlist: `useWishlist` · `useWishlistCount` ·
-`useAddToWishlist` · `useRemoveFromWishlist`. Favorites: `useFavorites` ·
-`useFavoritesCount` · `useIsFavorited` · `useAddToFavorites` ·
-`useRemoveFromFavorites`. Ratings: `useRateStorefrontProduct` ·
-`useRateStorefrontShop`. Seller: `useUpdateStorefrontProfile` ·
-`useCheckSlugAvailable` · `useUpdateStorefrontListing` ·
-`useUploadProductImage` · `useBusinessSocialLinks` /
-`useUpsertBusinessSocialLink` / `useDeleteBusinessSocialLink`.
-**API endpoints (BE):** `GET /storefront/discover` · `/storefront/categories`
-· `/storefront/facets` · `/storefront/shops` · `/storefront/{slug}` ·
-`/storefront/{slug}/products` · `/storefront/{slug}/products/{productSlug}` ·
-`POST /storefront/{slug}/ratings` · `POST
-/storefront/{slug}/products/{product}/ratings` · `POST
-/storefront/{slug}/orders` (throttle:storefront-orders) · `GET
-/storefront/my-orders` + `/{order}/sale` + `/{order}/invoice` +
-`/{order}/invoice/pdf` + `POST /{order}/cancel` + `DELETE /{order}` ·
-`/storefront/wishlist` (+ `POST`, `DELETE /by-product/{product}`) ·
-`/storefront/favorites` (+ `POST`, `DELETE /{business}`). Seller-side:
-`PATCH /businesses/storefront-profile` · `GET /businesses/slug-available` ·
-`PATCH /products/{id}/storefront-listing` · `POST /products/{id}/image` ·
-`/business-social-links` CRUD.
-**Route middleware (BE):** public catalog/shop routes have no auth; buyer
-auth-gated routes (orders, wishlist, favorites, ratings, place order) use
-`auth:sanctum`, with `throttle:60,1` on wishlist/favorites/ratings and
-`throttle:storefront-orders` on placing orders.
-**Key types (FE):** `StorefrontShop` (name, slug, description, logo, city,
-country, phone, email, currency, rating_avg/count, my_rating, category,
-social_links) · `StorefrontProduct` (slug, unit_price, compare_at_price,
-sale_price, discount_percent, unit, image_path, type product|service,
-stock_quantity, in_stock, availability, rating_avg/count, business) ·
-`MyStorefrontOrder` (order_number, status open|completed|invoiced|cancelled,
-total_amount, items, customer_name/phone, delivery_address/city, notes,
-shop_name/slug, currency, sale_id, receipt_number, invoice_id) ·
-`StorefrontCartBag` (per-shop bag: shop meta, items, notes, contact) ·
-`WishlistItem` (product) vs `FavoriteItem` (business) · Facets (business
-categories, countries/cities, currencies, product types, price bounds).
-**Notes:** multi-cart = one bag per shop slug, tabbed, submitted one at a time,
-persisted in localStorage (`custosell.storefront.cart.v1`), cleared on logout.
-Wishlist is for products (heart); favorites are for businesses (star); both
-server-backed and sign-in gated. Orders poll every 30s with a status-change
-chime. No theme/branding customization exists - shop look comes from the
-Business record (name, logo, description, contact, currency, social links).
 PUBLISHED TITLE: Facebook, WhatsApp, TikTok - on your shop page.
 SHORT-FORM VARIANT: Facebook, WhatsApp, TikTok
 PUBLISHED DESCRIPTION: Add your social links in settings and they appear on your public shop with brand icons - so customers can follow, message, and find you. Try free #custosell #storefront #onlineshop #ecommerce #Custosell #SmallBusiness
@@ -14691,7 +14632,66 @@
   - Screen-record clips: the Screen flow steps, trimmed to the script beats
   - Captions / subtitles: full on-screen captions exported as a caption file
   - Brand overlay / watermark: Custosell logo, corner placement
-  - Music: royalty-free background bed, low volume under the voiceover</t>
+  - Music: royalty-free background bed, low volume under the voiceover
+  - ---
+  - ## Technical reference (source of truth)
+  - **Screens (buyer):** `/discover` [M] (Businesses / Products tabs, infinite
+  - catalogs) · `/discover/shop/{slug}` [M] (shop catalog, filters, product modal,
+  - QR, social) · `/discover/my-orders` [M] (status tabs, cancel/delete, receipt,
+  - invoice) · `/discover/wishlist` [M] · `/discover/favorites` [M] · `/{@slug}`
+  - and `/{@slug}/p/{productSlug}` [M] (public share handles that redirect into the
+  - app). Seller setup lives in Settings -&gt; Sales channels (`BusinessStorefrontCard`,
+  - `ShopUsernameField`, QR download) and Inventory -&gt; products
+  - (`ProductStorefrontListingSection`, bulk list/unlist, image upload).
+  - **User actions (FE hooks):** Catalog: `useStorefrontShopsInfinite` ·
+  - `useStorefrontDiscoverInfinite` · `useStorefrontFacets` ·
+  - `useStorefrontCategories` · `useStorefrontShop` ·
+  - `useStorefrontShopProductsInfinite` · `useStorefrontShopProduct`. Orders:
+  - `useMyStorefrontOrdersList` (30s poll) · `useMyStorefrontOrdersCount` ·
+  - `usePlaceStorefrontOrder` · `useCancelMyStorefrontOrder` ·
+  - `useDeleteMyStorefrontOrder` · `fetchMyStorefrontOrderSale` ·
+  - `fetchMyStorefrontOrderInvoice`. Wishlist: `useWishlist` · `useWishlistCount` ·
+  - `useAddToWishlist` · `useRemoveFromWishlist`. Favorites: `useFavorites` ·
+  - `useFavoritesCount` · `useIsFavorited` · `useAddToFavorites` ·
+  - `useRemoveFromFavorites`. Ratings: `useRateStorefrontProduct` ·
+  - `useRateStorefrontShop`. Seller: `useUpdateStorefrontProfile` ·
+  - `useCheckSlugAvailable` · `useUpdateStorefrontListing` ·
+  - `useUploadProductImage` · `useBusinessSocialLinks` /
+  - `useUpsertBusinessSocialLink` / `useDeleteBusinessSocialLink`.
+  - **API endpoints (BE):** `GET /storefront/discover` · `/storefront/categories`
+  - · `/storefront/facets` · `/storefront/shops` · `/storefront/{slug}` ·
+  - `/storefront/{slug}/products` · `/storefront/{slug}/products/{productSlug}` ·
+  - `POST /storefront/{slug}/ratings` · `POST
+  - /storefront/{slug}/products/{product}/ratings` · `POST
+  - /storefront/{slug}/orders` (throttle:storefront-orders) · `GET
+  - /storefront/my-orders` + `/{order}/sale` + `/{order}/invoice` +
+  - `/{order}/invoice/pdf` + `POST /{order}/cancel` + `DELETE /{order}` ·
+  - `/storefront/wishlist` (+ `POST`, `DELETE /by-product/{product}`) ·
+  - `/storefront/favorites` (+ `POST`, `DELETE /{business}`). Seller-side:
+  - `PATCH /businesses/storefront-profile` · `GET /businesses/slug-available` ·
+  - `PATCH /products/{id}/storefront-listing` · `POST /products/{id}/image` ·
+  - `/business-social-links` CRUD.
+  - **Route middleware (BE):** public catalog/shop routes have no auth; buyer
+  - auth-gated routes (orders, wishlist, favorites, ratings, place order) use
+  - `auth:sanctum`, with `throttle:60,1` on wishlist/favorites/ratings and
+  - `throttle:storefront-orders` on placing orders.
+  - **Key types (FE):** `StorefrontShop` (name, slug, description, logo, city,
+  - country, phone, email, currency, rating_avg/count, my_rating, category,
+  - social_links) · `StorefrontProduct` (slug, unit_price, compare_at_price,
+  - sale_price, discount_percent, unit, image_path, type product|service,
+  - stock_quantity, in_stock, availability, rating_avg/count, business) ·
+  - `MyStorefrontOrder` (order_number, status open|completed|invoiced|cancelled,
+  - total_amount, items, customer_name/phone, delivery_address/city, notes,
+  - shop_name/slug, currency, sale_id, receipt_number, invoice_id) ·
+  - `StorefrontCartBag` (per-shop bag: shop meta, items, notes, contact) ·
+  - `WishlistItem` (product) vs `FavoriteItem` (business) · Facets (business
+  - categories, countries/cities, currencies, product types, price bounds).
+  - **Notes:** multi-cart = one bag per shop slug, tabbed, submitted one at a time,
+  - persisted in localStorage (`custosell.storefront.cart.v1`), cleared on logout.
+  - Wishlist is for products (heart); favorites are for businesses (star); both
+  - server-backed and sign-in gated. Orders poll every 30s with a status-change
+  - chime. No theme/branding customization exists - shop look comes from the
+  - Business record (name, logo, description, contact, currency, social links).</t>
         </is>
       </c>
       <c r="D236" s="5" t="n"/>
@@ -15619,86 +15619,6 @@
 DEMO DATA: Multiple branches with staff.
 CTA: Try free
 RELATED: [17-settings.md](./17-settings.md)
----
-## Technical reference (source of truth)
-**Screens:** `/hr` (index redirects to overview for full HR, attendance for
-limited HR) · `/hr/overview` [M] · `/hr/people` [M] + `/hr/people/{id}` [M]
-(detail editor incl. login section) · `/hr/departments` [M] ·
-`/hr/company-assets` [M] + `/hr/company-assets/{id}` [M] ·
-`/hr/attendance` [M] · `/hr/leave` [M] · `/hr/payroll` [M] +
-`/hr/payroll/runs/{id}` [M] · `/hr/talent` [M] (tabs: performance / onboarding
-/ reviews) · `/hr/transfers` [M] · `/hr/reports` [M] · `/hr/settings` [M]
-(audit log viewer). Full HR access = owner or staff with `hr_full`; limited HR
-users only get attendance, leave, and talent.
-**User actions (FE hooks):** Org: `useHrDepartments` / CRUD ·
-`useHrPositions` / CRUD. Employees: `useHrEmployees` · `useHrEmployee` ·
-`useCreateHrEmployee` · `useCreateHrEmployeeWithAccount` · `useHrAccountOptions`
-· `useUpdateHrEmployee` · `useDeleteHrEmployee` · `useLinkHrEmployeeUser` ·
-`useUnlinkHrEmployeeUser` · `useCreateHrEmployeeAccount` ·
-`useRemoveHrEmployeeAccount`. Attendance: `useHrAttendance` (register +
-events) · `useHrClock` · `useUpdateHrAttendanceDay` · `useImportHrTimesheets` ·
-`useHrPosShifts`. Leave: `useHrLeaveTypes` / CRUD · `useHrLeaveBalances` ·
-`useHrLeaveRequests` · `useCreateHrLeaveRequest` · `useApproveHrLeaveRequest` ·
-`useRejectHrLeaveRequest` · `useCancelHrLeaveRequest`. Payroll:
-`useHrSalaryStructures` / CRUD · `useHrCompensations` / create/delete ·
-`useHrPayRuns` · `useHrPayRun` · `useCreateHrPayRun` · `useUpdateHrPayRun` ·
-`useDeleteHrPayRun` · `useCalculateHrPayRun` · `useApproveHrPayRun` ·
-`usePostHrPayRun` · `useSettleHrPayRun` · `useRemitHrStatutory` ·
-`useVoidHrPayRun`. Talent: `useHrOnboardingTemplates` / CRUD ·
-`useHrOnboardingTasks` / create/update · `useHrReviews` / create/update ·
-`useHrPerformanceRoster` · `useHrPerformanceEmployee` ·
-`useHrPerformanceByUser` · `useSeedHrPerformanceReview`. Assets:
-`useHrCompanyAssets` · `useHrCompanyAsset` · `useCreateHrCompanyAsset` ·
-`useUpdateHrCompanyAssetCustody` · `useAssignHrCompanyAsset` ·
-`useTransferHrCompanyAsset` · `useReturnHrCompanyAsset` ·
-`useHrCompanyAssetAssignments` · `useHrCompanyAssetMaintenanceExpenses`.
-Reports: `useHrPayeReport` · `useHrNssfReport` · `useHrPayrollAffordability`
-(POST) · `useHrPayrollAffordabilityMutation` · `useHrAuditLogs`.
-**API endpoints (BE):** `/hr/departments` CRUD · `/hr/positions` CRUD ·
-`/hr/employees` + `/hr/employees/sync-staff` + `/hr/employees/with-account` +
-`/hr/account-options` + `/{id}` CRUD + `/{id}/link-user` + `/{id}/unlink-user`
-+ `/{id}/create-account` + `/{id}/remove-account` · `/hr/attendance/clock` +
-`/hr/attendance/events` + `/hr/attendance/register` + `/hr/attendance/days`
-(PUT) + `/hr/attendance/import-timesheets` + `/hr/attendance/pos-shifts` ·
-`/hr/leave/types` CRUD + `/hr/leave/balances` + `/hr/leave/balances/ensure` +
-`/hr/leave/requests` + `/{id}/approve` + `/{id}/reject` + `/{id}/cancel` ·
-`/hr/payroll/structures` CRUD + `/hr/payroll/compensations` + `/hr/payroll/
-pay-runs` CRUD + `/{id}/calculate` + `/{id}/approve` + `/{id}/post` +
-`/{id}/settle` + `/{id}/remit-statutory` + `/{id}/void` ·
-`/hr/talent/onboarding-templates` CRUD + `/hr/talent/onboarding-tasks` +
-`/hr/talent/onboarding/assign` + `/hr/talent/reviews` +
-`/hr/talent/performance` + `/hr/talent/performance/employees/{id}` +
-`/hr/talent/performance/by-user/{id}` + `/hr/talent/performance/employees/
-{id}/seed-review` · `/hr/reports/paye-schedule` + `/hr/reports/nssf-schedule`
-+ `/hr/reports/payroll-affordability` (POST) + `/hr/audit-logs` ·
-`/hr/company-assets` CRUD + `/{id}/assign` + `/{id}/transfer` + `/{id}/return`
-+ `/{id}/assignments` + `/{id}/maintenance-expenses`. Cross-module:
-`/staff-transfers` CRUD (settings module), `/users`, `/locations`.
-**Route middleware (BE):** all HR routes use `auth:sanctum` ·
-`business.active` · `subscription.active` · `module:hr`. Sensitive routes
-(org, employee writes, attendance corrections, leave decisions, all payroll,
-talent templates/reviews, reports, assets) additionally require `hr.full`
-middleware; clock, events, register, leave request/cancel, and onboarding-task
-updates are self-service for limited users. Online-only module.
-**Key statuses (FE):** `EmployeeStatus` = onboarding | active | on_leave |
-terminated · `EmploymentType` = full_time | part_time | contract | casual ·
-`PayRunStatus` = draft | calculated | approved | posted | void ·
-`AttendanceEventType` = clock_in | clock_out | break_start | break_end ·
-`AttendanceDayStatus` = present | absent | leave | holiday · `LeaveRequestStatus`
-= pending | approved | rejected | cancelled · `OnboardingTaskStatus` = pending
-| done | skipped · `ReviewStatus` = draft | submitted | completed ·
-`PerformanceVerdict` = on_track | at_risk | behind | no_data | unlinked ·
-`AssetCategory` = laptop | phone | furniture | vehicle | other · `AssetCondition`
-= new | good | fair | poor | retired.
-**Notes:** pay run lifecycle writes accounting journals (accrual Dr 6101 / Cr
-2110-2112, settlement Dr Salaries Payable / Cr Bank 1102, statutory remit Dr
-PAYE + NSSF payable / Cr Bank) and invalidates HR statutory reports on
-post/void. Company assets share the accounting FixedAsset entity (book value
-synced). Performance is computed from Pipeline leads + Project tasks + board
-goals, and seeded review drafts carry that snapshot. Payroll affordability
-defaults to a 3-month horizon and supports a hire what-if (basic salary,
-allowances, deductions, start month offset). Payslips are embedded on pay-run
-lines (no dedicated endpoint yet).
 PUBLISHED TITLE: Move staff between branches, tracked.
 SHORT-FORM VARIANT: Move staff between branches
 PUBLISHED DESCRIPTION: Transfer a staff member from one branch to another - permanent or temporary - and keep the whole history visible with branch headcount overviews. Try free #custosell #hr #payroll #employees #Custosell #SmallBusiness
@@ -15708,7 +15628,87 @@
   - Screen-record clips: the Screen flow steps, trimmed to the script beats
   - Captions / subtitles: full on-screen captions exported as a caption file
   - Brand overlay / watermark: Custosell logo, corner placement
-  - Music: royalty-free background bed, low volume under the voiceover</t>
+  - Music: royalty-free background bed, low volume under the voiceover
+  - ---
+  - ## Technical reference (source of truth)
+  - **Screens:** `/hr` (index redirects to overview for full HR, attendance for
+  - limited HR) · `/hr/overview` [M] · `/hr/people` [M] + `/hr/people/{id}` [M]
+  - (detail editor incl. login section) · `/hr/departments` [M] ·
+  - `/hr/company-assets` [M] + `/hr/company-assets/{id}` [M] ·
+  - `/hr/attendance` [M] · `/hr/leave` [M] · `/hr/payroll` [M] +
+  - `/hr/payroll/runs/{id}` [M] · `/hr/talent` [M] (tabs: performance / onboarding
+  - / reviews) · `/hr/transfers` [M] · `/hr/reports` [M] · `/hr/settings` [M]
+  - (audit log viewer). Full HR access = owner or staff with `hr_full`; limited HR
+  - users only get attendance, leave, and talent.
+  - **User actions (FE hooks):** Org: `useHrDepartments` / CRUD ·
+  - `useHrPositions` / CRUD. Employees: `useHrEmployees` · `useHrEmployee` ·
+  - `useCreateHrEmployee` · `useCreateHrEmployeeWithAccount` · `useHrAccountOptions`
+  - · `useUpdateHrEmployee` · `useDeleteHrEmployee` · `useLinkHrEmployeeUser` ·
+  - `useUnlinkHrEmployeeUser` · `useCreateHrEmployeeAccount` ·
+  - `useRemoveHrEmployeeAccount`. Attendance: `useHrAttendance` (register +
+  - events) · `useHrClock` · `useUpdateHrAttendanceDay` · `useImportHrTimesheets` ·
+  - `useHrPosShifts`. Leave: `useHrLeaveTypes` / CRUD · `useHrLeaveBalances` ·
+  - `useHrLeaveRequests` · `useCreateHrLeaveRequest` · `useApproveHrLeaveRequest` ·
+  - `useRejectHrLeaveRequest` · `useCancelHrLeaveRequest`. Payroll:
+  - `useHrSalaryStructures` / CRUD · `useHrCompensations` / create/delete ·
+  - `useHrPayRuns` · `useHrPayRun` · `useCreateHrPayRun` · `useUpdateHrPayRun` ·
+  - `useDeleteHrPayRun` · `useCalculateHrPayRun` · `useApproveHrPayRun` ·
+  - `usePostHrPayRun` · `useSettleHrPayRun` · `useRemitHrStatutory` ·
+  - `useVoidHrPayRun`. Talent: `useHrOnboardingTemplates` / CRUD ·
+  - `useHrOnboardingTasks` / create/update · `useHrReviews` / create/update ·
+  - `useHrPerformanceRoster` · `useHrPerformanceEmployee` ·
+  - `useHrPerformanceByUser` · `useSeedHrPerformanceReview`. Assets:
+  - `useHrCompanyAssets` · `useHrCompanyAsset` · `useCreateHrCompanyAsset` ·
+  - `useUpdateHrCompanyAssetCustody` · `useAssignHrCompanyAsset` ·
+  - `useTransferHrCompanyAsset` · `useReturnHrCompanyAsset` ·
+  - `useHrCompanyAssetAssignments` · `useHrCompanyAssetMaintenanceExpenses`.
+  - Reports: `useHrPayeReport` · `useHrNssfReport` · `useHrPayrollAffordability`
+  - (POST) · `useHrPayrollAffordabilityMutation` · `useHrAuditLogs`.
+  - **API endpoints (BE):** `/hr/departments` CRUD · `/hr/positions` CRUD ·
+  - `/hr/employees` + `/hr/employees/sync-staff` + `/hr/employees/with-account` +
+  - `/hr/account-options` + `/{id}` CRUD + `/{id}/link-user` + `/{id}/unlink-user`
+  - + `/{id}/create-account` + `/{id}/remove-account` · `/hr/attendance/clock` +
+  - `/hr/attendance/events` + `/hr/attendance/register` + `/hr/attendance/days`
+  - (PUT) + `/hr/attendance/import-timesheets` + `/hr/attendance/pos-shifts` ·
+  - `/hr/leave/types` CRUD + `/hr/leave/balances` + `/hr/leave/balances/ensure` +
+  - `/hr/leave/requests` + `/{id}/approve` + `/{id}/reject` + `/{id}/cancel` ·
+  - `/hr/payroll/structures` CRUD + `/hr/payroll/compensations` + `/hr/payroll/
+  - pay-runs` CRUD + `/{id}/calculate` + `/{id}/approve` + `/{id}/post` +
+  - `/{id}/settle` + `/{id}/remit-statutory` + `/{id}/void` ·
+  - `/hr/talent/onboarding-templates` CRUD + `/hr/talent/onboarding-tasks` +
+  - `/hr/talent/onboarding/assign` + `/hr/talent/reviews` +
+  - `/hr/talent/performance` + `/hr/talent/performance/employees/{id}` +
+  - `/hr/talent/performance/by-user/{id}` + `/hr/talent/performance/employees/
+  - {id}/seed-review` · `/hr/reports/paye-schedule` + `/hr/reports/nssf-schedule`
+  - + `/hr/reports/payroll-affordability` (POST) + `/hr/audit-logs` ·
+  - `/hr/company-assets` CRUD + `/{id}/assign` + `/{id}/transfer` + `/{id}/return`
+  - + `/{id}/assignments` + `/{id}/maintenance-expenses`. Cross-module:
+  - `/staff-transfers` CRUD (settings module), `/users`, `/locations`.
+  - **Route middleware (BE):** all HR routes use `auth:sanctum` ·
+  - `business.active` · `subscription.active` · `module:hr`. Sensitive routes
+  - (org, employee writes, attendance corrections, leave decisions, all payroll,
+  - talent templates/reviews, reports, assets) additionally require `hr.full`
+  - middleware; clock, events, register, leave request/cancel, and onboarding-task
+  - updates are self-service for limited users. Online-only module.
+  - **Key statuses (FE):** `EmployeeStatus` = onboarding | active | on_leave |
+  - terminated · `EmploymentType` = full_time | part_time | contract | casual ·
+  - `PayRunStatus` = draft | calculated | approved | posted | void ·
+  - `AttendanceEventType` = clock_in | clock_out | break_start | break_end ·
+  - `AttendanceDayStatus` = present | absent | leave | holiday · `LeaveRequestStatus`
+  - = pending | approved | rejected | cancelled · `OnboardingTaskStatus` = pending
+  - | done | skipped · `ReviewStatus` = draft | submitted | completed ·
+  - `PerformanceVerdict` = on_track | at_risk | behind | no_data | unlinked ·
+  - `AssetCategory` = laptop | phone | furniture | vehicle | other · `AssetCondition`
+  - = new | good | fair | poor | retired.
+  - **Notes:** pay run lifecycle writes accounting journals (accrual Dr 6101 / Cr
+  - 2110-2112, settlement Dr Salaries Payable / Cr Bank 1102, statutory remit Dr
+  - PAYE + NSSF payable / Cr Bank) and invalidates HR statutory reports on
+  - post/void. Company assets share the accounting FixedAsset entity (book value
+  - synced). Performance is computed from Pipeline leads + Project tasks + board
+  - goals, and seeded review drafts carry that snapshot. Payroll affordability
+  - defaults to a 3-month horizon and supports a hire what-if (basic salary,
+  - allowances, deductions, start month offset). Payslips are embedded on pay-run
+  - lines (no dedicated endpoint yet).</t>
         </is>
       </c>
       <c r="D252" s="5" t="n"/>
@@ -16161,44 +16161,6 @@
 DEMO DATA: Recurring products/services with prices.
 CTA: Try free
 RELATED: [05-inventory-products.md](./05-inventory-products.md)
----
-## Technical reference (source of truth)
-**Screens:** `/forecasting` [M] (INDEX -&gt; overview: cash ladder, burn breakdown,
-budget vs actual, coverage snapshot, quick links) · `/forecasting/budgets` [M]
-(year budget list + create) · `/forecasting/budgets/{id}` [M] (lines with
-justify/approve/roll + snapshots) · `/forecasting/kpis` [M] (retail + saas) ·
-`/forecasting/scenarios` [M] (what-if create/list/run)
-**User actions (FE hooks):** `useForecastingOverview` · `useCashForecast` ·
-`useBudgetVsActual` · `useForecastKpis` · `useForecastBudgets` ·
-`useForecastBudget` · `useCreateForecastBudget` · `useUpdateForecastBudget` ·
-`useDeleteForecastBudget` · `useCreateForecastBudgetLine` ·
-`useUpdateForecastBudgetLine` · `useDeleteForecastBudgetLine` ·
-`useJustifyForecastBudgetLine` · `useApproveForecastBudgetLine` ·
-`useRollForecastBudget` · `useForecastSnapshots` · `useForecastScenarios` ·
-`useForecastScenario` · `useCreateForecastScenario` ·
-`useUpdateForecastScenario` · `useDeleteForecastScenario` ·
-`useRunForecastScenario`
-**API endpoints (BE):** `GET /forecasting/overview` · `GET
-/forecasting/cash-forecast` · `GET /forecasting/budget-vs-actual` · `GET
-/forecasting/kpis` · `/forecasting/budgets` CRUD + `/{id}/lines` CRUD +
-`/{id}/lines/{lineId}/justify` + `/{id}/lines/{lineId}/approve` + `/{id}/roll`
-· `GET /forecasting/snapshots` · `/forecasting/scenarios` CRUD +
-`/{id}/run`
-**Route middleware (BE):** `auth:sanctum` · `business.active` ·
-`subscription.active` · `module:forecasting` (module must be enabled)
-**Key types (FE):** `ForecastCoverageStatus` = healthy | tight | critical |
-unknown · `ForecastBudgetStatus` = draft | active | archived ·
-`ForecastZbbStatus` = draft | justified | approved · `ForecastBvaStatus` = over
-| under | on_track · `ForecastKpiMode` = auto | retail | saas · `CashForecast`
-(cash, liabilities incl payroll/PAYE/NSSF payable, burn from HR payroll
-affordability + trailing opex, assumed monthly inflow from trailing 30d net
-sales, runway coverage, month cash ladder rows with can_cover) ·
-`BudgetVsActual` (per-category budget/actual/variance/status) · `ForecastBudget`
-+ `ForecastBudgetLine` (label, amount, justification, zbb_status) ·
-`ForecastSnapshot` (budget lines + YTD expense actuals captured on roll) ·
-`ForecastKpis` (retail: pulse/CAC/LTV/churn; saas: MRR/ARR/subscribers) ·
-`ForecastScenario` + `ForecastScenarioRun` (baseline + scenario forecast +
-delta)
 PUBLISHED TITLE: Sell recurring? See MRR and ARR proxies.
 SHORT-FORM VARIANT: Sell recurring? See MRR and ARR proxies.
 PUBLISHED DESCRIPTION: Mark products or services as recurring and the KPIs page shows MRR, ARR, active subscribers, and average recurring price as simple proxies from your own catalog. Try free #custosell #forecasting #budget #cashrunway #Custosell #SmallBusiness
@@ -16208,7 +16170,45 @@
   - Screen-record clips: the Screen flow steps, trimmed to the script beats
   - Captions / subtitles: full on-screen captions exported as a caption file
   - Brand overlay / watermark: Custosell logo, corner placement
-  - Music: royalty-free background bed, low volume under the voiceover</t>
+  - Music: royalty-free background bed, low volume under the voiceover
+  - ---
+  - ## Technical reference (source of truth)
+  - **Screens:** `/forecasting` [M] (INDEX -&gt; overview: cash ladder, burn breakdown,
+  - budget vs actual, coverage snapshot, quick links) · `/forecasting/budgets` [M]
+  - (year budget list + create) · `/forecasting/budgets/{id}` [M] (lines with
+  - justify/approve/roll + snapshots) · `/forecasting/kpis` [M] (retail + saas) ·
+  - `/forecasting/scenarios` [M] (what-if create/list/run)
+  - **User actions (FE hooks):** `useForecastingOverview` · `useCashForecast` ·
+  - `useBudgetVsActual` · `useForecastKpis` · `useForecastBudgets` ·
+  - `useForecastBudget` · `useCreateForecastBudget` · `useUpdateForecastBudget` ·
+  - `useDeleteForecastBudget` · `useCreateForecastBudgetLine` ·
+  - `useUpdateForecastBudgetLine` · `useDeleteForecastBudgetLine` ·
+  - `useJustifyForecastBudgetLine` · `useApproveForecastBudgetLine` ·
+  - `useRollForecastBudget` · `useForecastSnapshots` · `useForecastScenarios` ·
+  - `useForecastScenario` · `useCreateForecastScenario` ·
+  - `useUpdateForecastScenario` · `useDeleteForecastScenario` ·
+  - `useRunForecastScenario`
+  - **API endpoints (BE):** `GET /forecasting/overview` · `GET
+  - /forecasting/cash-forecast` · `GET /forecasting/budget-vs-actual` · `GET
+  - /forecasting/kpis` · `/forecasting/budgets` CRUD + `/{id}/lines` CRUD +
+  - `/{id}/lines/{lineId}/justify` + `/{id}/lines/{lineId}/approve` + `/{id}/roll`
+  - · `GET /forecasting/snapshots` · `/forecasting/scenarios` CRUD +
+  - `/{id}/run`
+  - **Route middleware (BE):** `auth:sanctum` · `business.active` ·
+  - `subscription.active` · `module:forecasting` (module must be enabled)
+  - **Key types (FE):** `ForecastCoverageStatus` = healthy | tight | critical |
+  - unknown · `ForecastBudgetStatus` = draft | active | archived ·
+  - `ForecastZbbStatus` = draft | justified | approved · `ForecastBvaStatus` = over
+  - | under | on_track · `ForecastKpiMode` = auto | retail | saas · `CashForecast`
+  - (cash, liabilities incl payroll/PAYE/NSSF payable, burn from HR payroll
+  - affordability + trailing opex, assumed monthly inflow from trailing 30d net
+  - sales, runway coverage, month cash ladder rows with can_cover) ·
+  - `BudgetVsActual` (per-category budget/actual/variance/status) · `ForecastBudget`
+  - + `ForecastBudgetLine` (label, amount, justification, zbb_status) ·
+  - `ForecastSnapshot` (budget lines + YTD expense actuals captured on roll) ·
+  - `ForecastKpis` (retail: pulse/CAC/LTV/churn; saas: MRR/ARR/subscribers) ·
+  - `ForecastScenario` + `ForecastScenarioRun` (baseline + scenario forecast +
+  - delta)</t>
         </is>
       </c>
       <c r="D260" s="5" t="n"/>
@@ -16663,62 +16663,6 @@
 DEMO DATA: A payment in pending status.
 CTA: Try free
 RELATED: [16-subscriptions-billing.md](./16-subscriptions-billing.md)
----
-## Technical reference (source of truth)
-**Screens:** `/settings/subscription` [M] (Plans + History tabs; shows
-available promo credit banner). Plans tab: current plan banner (status, billing
-cycle, next bill or trial end, setup fee status, payment action message, Renew
-Early), monthly/yearly toggle, plan cards with action buttons, feature
-comparison table, limits table. History tab: payment/change/credit timeline with
-receipt download + email + sync payment. Modals: UpgradeFlowModal,
-SubscriptionPaymentModal, BillingCycleSwitchModal, BillingCyclePaymentModal,
-RenewTopUpModal, EmailReceiptModal. Related UI: PlanCard, PlanUsageSection,
-PendingPaymentNotice, PlansTab in onboarding (ROUTES.ONBOARDING).
-**User actions (FE hooks):** `useActivePlans` (GET /plans/active) ·
-`useSubscribe` (POST /subscriptions/subscribe) · `useUpgradeQuote` (GET
-/subscriptions/{id}/proration-quote) · `useUpgrade` (POST
-/subscriptions/{id}/upgrade, effective immediate) · `useDowngrade` (POST
-/subscriptions/{id}/downgrade, effective end_of_period) ·
-`useSubscriptionChanges` (GET /subscriptions/{id}/changes) ·
-`useCancelScheduledChange` (POST /subscriptions/{id}/cancel-change) ·
-`useChangeBillingCycle` (POST /subscriptions/{id}/billing-cycle) ·
-`useInitiatePayment` (POST /billing/payments/initiate) ·
-`useInitiateOnboardingPayment` · `useConfirmPayment` (POST
-/billing/payments/{id}/confirm) · `useBillingPayment` (GET
-/billing/payments/{id}, 3s poll) · `useBillingHistory` (GET /billing/history) ·
-`downloadReceiptPdf` (GET /billing/payments/{id}/receipt) · `useEmailReceipt`
-(POST /billing/payments/{id}/receipt/email) · `useReferralEarnings`
-(available_credit banner). Also `useProfile` refresh after payment, and the
-platform-side `usePlans`/`useSubscriptions` (admin registry).
-**API endpoints (BE):** `/plans/active` + `/plans` (apiResource) ·
-`/subscriptions/current` · `/subscriptions/subscribe` ·
-`/subscriptions/{id}/cancel` · `/subscriptions/{id}/upgrade` ·
-`/subscriptions/{id}/downgrade` · `/subscriptions/{id}/proration-quote` ·
-`/subscriptions/{id}/changes` · `/subscriptions/{id}/cancel-change` ·
-`/subscriptions/{id}/billing-cycle` · `/subscriptions/access` ·
-`/billing/payments` · `/billing/payments/{id}` ·
-`/billing/payments/{id}/receipt` · `/billing/payments/{id}/receipt/email` ·
-`/billing/history` · `/billing/payments/initiate` ·
-`/billing/payments/{id}/confirm` · gateway webhooks/callback (PesaPal):
-`/billing/gateway/pesapal/webhook` + `/billing/gateway/pesapal/callback` +
-`/billing/gateway/pesapal/ipn`. Scheduled jobs (console): expire-trials,
-renew, suspend-past-due, cancel-at-period-end (02:00-02:45 daily).
-**Route middleware (BE):** business-facing subscription + billing routes use
-`auth:sanctum` + `business.active`; platform-only subscription registry
-(index/show) requires `platform:platform.businesses.view`. Generic plan/status
-mutation by owners is intentionally NOT exposed - changes happen only through
-payment-approved flows (initiate + confirm) or the platform.
-**Key concepts (FE):** `PlanActionType` = subscribe | resubscribe | reactivate
-| upgrade | downgrade | current | pay_onboarding | renew | renew_early |
-subscribe_early, resolved by a matrix over subscription status
-(none/trial_paid/trial_unpaid/active/past_due/suspended/expired/cancelled) x
-plan relation (current/higher/lower). `PaymentType` = subscription | onboarding
-| renewal | upgrade_proration | topup. `SubscriptionInfo` carries plan_id,
-status, billing_cycle, next_billing_date, trial_ends_at, onboarding_fee_paid,
-payment_action. History item types = payment | change | credit with statuses
-applied/pending/cancelled/failed/refunded/completed/successful. Payment
-currency: UGX/KES/TZS via PesaPal, otherwise USD. Billing history lives on the
-profile (auth store) and refreshes after confirmed payments.
 PUBLISHED TITLE: Paid but still pending? Sync it.
 SHORT-FORM VARIANT: Paid but still pending? Sync it.
 PUBLISHED DESCRIPTION: When a payment shows pending, tap Sync payment to re-check with the provider and confirm the real status - so your subscription updates immediately. Try free #custosell #subscription #billing #plans #Custosell #SmallBusiness
@@ -16728,7 +16672,63 @@
   - Screen-record clips: the Screen flow steps, trimmed to the script beats
   - Captions / subtitles: full on-screen captions exported as a caption file
   - Brand overlay / watermark: Custosell logo, corner placement
-  - Music: royalty-free background bed, low volume under the voiceover</t>
+  - Music: royalty-free background bed, low volume under the voiceover
+  - ---
+  - ## Technical reference (source of truth)
+  - **Screens:** `/settings/subscription` [M] (Plans + History tabs; shows
+  - available promo credit banner). Plans tab: current plan banner (status, billing
+  - cycle, next bill or trial end, setup fee status, payment action message, Renew
+  - Early), monthly/yearly toggle, plan cards with action buttons, feature
+  - comparison table, limits table. History tab: payment/change/credit timeline with
+  - receipt download + email + sync payment. Modals: UpgradeFlowModal,
+  - SubscriptionPaymentModal, BillingCycleSwitchModal, BillingCyclePaymentModal,
+  - RenewTopUpModal, EmailReceiptModal. Related UI: PlanCard, PlanUsageSection,
+  - PendingPaymentNotice, PlansTab in onboarding (ROUTES.ONBOARDING).
+  - **User actions (FE hooks):** `useActivePlans` (GET /plans/active) ·
+  - `useSubscribe` (POST /subscriptions/subscribe) · `useUpgradeQuote` (GET
+  - /subscriptions/{id}/proration-quote) · `useUpgrade` (POST
+  - /subscriptions/{id}/upgrade, effective immediate) · `useDowngrade` (POST
+  - /subscriptions/{id}/downgrade, effective end_of_period) ·
+  - `useSubscriptionChanges` (GET /subscriptions/{id}/changes) ·
+  - `useCancelScheduledChange` (POST /subscriptions/{id}/cancel-change) ·
+  - `useChangeBillingCycle` (POST /subscriptions/{id}/billing-cycle) ·
+  - `useInitiatePayment` (POST /billing/payments/initiate) ·
+  - `useInitiateOnboardingPayment` · `useConfirmPayment` (POST
+  - /billing/payments/{id}/confirm) · `useBillingPayment` (GET
+  - /billing/payments/{id}, 3s poll) · `useBillingHistory` (GET /billing/history) ·
+  - `downloadReceiptPdf` (GET /billing/payments/{id}/receipt) · `useEmailReceipt`
+  - (POST /billing/payments/{id}/receipt/email) · `useReferralEarnings`
+  - (available_credit banner). Also `useProfile` refresh after payment, and the
+  - platform-side `usePlans`/`useSubscriptions` (admin registry).
+  - **API endpoints (BE):** `/plans/active` + `/plans` (apiResource) ·
+  - `/subscriptions/current` · `/subscriptions/subscribe` ·
+  - `/subscriptions/{id}/cancel` · `/subscriptions/{id}/upgrade` ·
+  - `/subscriptions/{id}/downgrade` · `/subscriptions/{id}/proration-quote` ·
+  - `/subscriptions/{id}/changes` · `/subscriptions/{id}/cancel-change` ·
+  - `/subscriptions/{id}/billing-cycle` · `/subscriptions/access` ·
+  - `/billing/payments` · `/billing/payments/{id}` ·
+  - `/billing/payments/{id}/receipt` · `/billing/payments/{id}/receipt/email` ·
+  - `/billing/history` · `/billing/payments/initiate` ·
+  - `/billing/payments/{id}/confirm` · gateway webhooks/callback (PesaPal):
+  - `/billing/gateway/pesapal/webhook` + `/billing/gateway/pesapal/callback` +
+  - `/billing/gateway/pesapal/ipn`. Scheduled jobs (console): expire-trials,
+  - renew, suspend-past-due, cancel-at-period-end (02:00-02:45 daily).
+  - **Route middleware (BE):** business-facing subscription + billing routes use
+  - `auth:sanctum` + `business.active`; platform-only subscription registry
+  - (index/show) requires `platform:platform.businesses.view`. Generic plan/status
+  - mutation by owners is intentionally NOT exposed - changes happen only through
+  - payment-approved flows (initiate + confirm) or the platform.
+  - **Key concepts (FE):** `PlanActionType` = subscribe | resubscribe | reactivate
+  - | upgrade | downgrade | current | pay_onboarding | renew | renew_early |
+  - subscribe_early, resolved by a matrix over subscription status
+  - (none/trial_paid/trial_unpaid/active/past_due/suspended/expired/cancelled) x
+  - plan relation (current/higher/lower). `PaymentType` = subscription | onboarding
+  - | renewal | upgrade_proration | topup. `SubscriptionInfo` carries plan_id,
+  - status, billing_cycle, next_billing_date, trial_ends_at, onboarding_fee_paid,
+  - payment_action. History item types = payment | change | credit with statuses
+  - applied/pending/cancelled/failed/refunded/completed/successful. Payment
+  - currency: UGX/KES/TZS via PesaPal, otherwise USD. Billing history lives on the
+  - profile (auth store) and refreshes after confirmed payments.</t>
         </is>
       </c>
       <c r="D268" s="5" t="n"/>
@@ -16893,7 +16893,7 @@
   - Beat 1 (Hook): "Referrals are only fun when you can watch them pay off."
   - Beat 2 (Problem): "Rewards nobody can see feel fake."
   - Beat 3 (Action): Referral Dashboard -&gt; Wins tab -&gt; Referrals / Earned /
-  - Paid / Bal cards -&gt; Referred Businesses list -&gt; Payout History.
+  - Paid / Balance cards -&gt; Referred Businesses list -&gt; Payout History.
   - Beat 4 (Aha): "Every referral shows its status and reward - pending, active,
   - or rewarded."
   - Beat 5 (CTA): "Check your dashboard at custosell.com."
@@ -17091,39 +17091,6 @@
 DEMO DATA: A business with an active referral program.
 CTA: Try free
 RELATED: [20-referrals-credits.md](./20-referrals-credits.md)
----
-## Technical reference (source of truth)
-**Screens:** Navbar `Refer &amp; Earn` dropdown (ReferralDropdown) ·
-`/account/referrals` Referral Dashboard (code card + Wins / Policy / Help tabs)
-· signup `ReferralEntryPage` ("Have a referral code?")
-**User actions (FE hooks):** `useReferralEarnings` (GET `/referrals/earnings/me`)
-· `useGenerateReferralCode` (POST `/referral-codes`, owner business) ·
-`useApplyReferralCode` (POST `/referrals/apply`) ·
-`useValidateReferralCode` (GET `/referral-codes/validate`) ·
-`usePaymentInfo` + `useUpdatePaymentInfo` (GET/PUT `/account/payment-info`) ·
-`usePayoutHistory` (GET `/payouts/my-history`)
-**Referral earnings fields:** `referral_code` · `is_sales_rep` ·
-`commission_rate` / `commission_type` · `total_earned` · `rewards_paid` ·
-`commission_earned` / `commission_paid` · `total_referrals` ·
-`available_credit` / `business_credit` / `user_credit` · `referrals[]`
-(referred business, status pending/active/rewarded, reward_amount,
-commission_earned)
-**API endpoints (BE):** `referrals.php` (auth:sanctum + business.active):
-`GET /referrals` · `GET /referrals/{id}` · `GET /referrals/business/{businessId}`
-· `GET /referrals/code/{codeId}` · `GET /referrals/earnings/me` ·
-`POST /referrals/apply` · `GET|PUT /account/payment-info` ·
-`GET /payouts/my-history` · `referral-codes.php`: `GET /referral-codes/validate`
-(public) + apiResource `referral-codes` · `credits.php`:
-`GET /credits/balance` + `GET /credits/history` (auth:sanctum +
-business.active) · `sales-reps.php` (auth:sanctum + business.active +
-subscription.active): apiResource `sales-reps` · `GET /sales-reps/import-template`
-· `POST /sales-reps/import` · `GET /sales-reps/earnings/all` ·
-`GET /sales-reps/earnings/mine` · `GET /sales-reps/{id}/earnings` ·
-`GET /sales-reps/{id}/payouts` · `POST /sales-reps/{id}/payouts`
-**Platform admin (not end-user):** `/platform/sales-reps` - manage sales reps
-(add/edit with commission rate + type + referee discount + active toggle,
-remove blocked while unpaid commission remains, CSV import from template, record
-payouts now or scheduled with method/notes/attachments).
 PUBLISHED TITLE: How Custosell referrals work - the simple version.
 SHORT-FORM VARIANT: How Custosell referrals work
 PUBLISHED DESCRIPTION: Understand the Custosell referral program in plain language: how rewards are calculated, whether there are limits, when payouts happen, and what is not allowed. One referral code per referred business, rewards based on the plan actually paid. Try free #custosell #referrals #credits #rewards #Custosell #SmallBusiness
@@ -17133,7 +17100,40 @@
   - Screen-record clips: the Screen flow steps, trimmed to the script beats
   - Captions / subtitles: full on-screen captions exported as a caption file
   - Brand overlay / watermark: Custosell logo, corner placement
-  - Music: royalty-free background bed, low volume under the voiceover</t>
+  - Music: royalty-free background bed, low volume under the voiceover
+  - ---
+  - ## Technical reference (source of truth)
+  - **Screens:** Navbar `Refer &amp; Earn` dropdown (ReferralDropdown) ·
+  - `/account/referrals` Referral Dashboard (code card + Wins / Policy / Help tabs)
+  - · signup `ReferralEntryPage` ("Have a referral code?")
+  - **User actions (FE hooks):** `useReferralEarnings` (GET `/referrals/earnings/me`)
+  - · `useGenerateReferralCode` (POST `/referral-codes`, owner business) ·
+  - `useApplyReferralCode` (POST `/referrals/apply`) ·
+  - `useValidateReferralCode` (GET `/referral-codes/validate`) ·
+  - `usePaymentInfo` + `useUpdatePaymentInfo` (GET/PUT `/account/payment-info`) ·
+  - `usePayoutHistory` (GET `/payouts/my-history`)
+  - **Referral earnings fields:** `referral_code` · `is_sales_rep` ·
+  - `commission_rate` / `commission_type` · `total_earned` · `rewards_paid` ·
+  - `commission_earned` / `commission_paid` · `total_referrals` ·
+  - `available_credit` / `business_credit` / `user_credit` · `referrals[]`
+  - (referred business, status pending/active/rewarded, reward_amount,
+  - commission_earned)
+  - **API endpoints (BE):** `referrals.php` (auth:sanctum + business.active):
+  - `GET /referrals` · `GET /referrals/{id}` · `GET /referrals/business/{businessId}`
+  - · `GET /referrals/code/{codeId}` · `GET /referrals/earnings/me` ·
+  - `POST /referrals/apply` · `GET|PUT /account/payment-info` ·
+  - `GET /payouts/my-history` · `referral-codes.php`: `GET /referral-codes/validate`
+  - (public) + apiResource `referral-codes` · `credits.php`:
+  - `GET /credits/balance` + `GET /credits/history` (auth:sanctum +
+  - business.active) · `sales-reps.php` (auth:sanctum + business.active +
+  - subscription.active): apiResource `sales-reps` · `GET /sales-reps/import-template`
+  - · `POST /sales-reps/import` · `GET /sales-reps/earnings/all` ·
+  - `GET /sales-reps/earnings/mine` · `GET /sales-reps/{id}/earnings` ·
+  - `GET /sales-reps/{id}/payouts` · `POST /sales-reps/{id}/payouts`
+  - **Platform admin (not end-user):** `/platform/sales-reps` - manage sales reps
+  - (add/edit with commission rate + type + referee discount + active toggle,
+  - remove blocked while unpaid commission remains, CSV import from template, record
+  - payouts now or scheduled with method/notes/attachments).</t>
         </is>
       </c>
       <c r="D274" s="5" t="n"/>
@@ -17351,35 +17351,6 @@
 DEMO DATA: A business account.
 CTA: Try free
 RELATED: [03-sales-pos.md](./03-sales-pos.md)
----
-## Technical reference (source of truth)
-**Screens:** `/notifications` [M] (modules/notifications/NotificationsPage) -
-inbox with All/Unread filters, open/read, mark-all-read, delete
-single/selected/all; the navbar bell (HeaderNotifications) shows the unread
-count; PushNotificationsCard and OrderSoundCard live at the top of the inbox.
-**User actions (FE hooks):** `useNotifications` (paginated, `per_page`,
-`unread_only`) · `useNotificationUnreadCount` · `useMarkNotificationRead` ·
-`useMarkAllNotificationsRead` · `useDeleteNotification` ·
-`useBulkDeleteNotifications` · `useDeleteAllNotifications` · `useWebPush`
-(toggle + status via `fetchWebPushStatus` / `storePushSubscription` /
-`removePushSubscription`) · `useSoundPreferences` (`orderSound`,
-`bigOrderThreshold`).
-**API endpoints (BE):** `GET /notifications` · `GET /notifications/unread-count`
-· `PATCH /notifications/read-all` · `PATCH /notifications/{id}/read` ·
-`DELETE /notifications/{id}` · `POST /notifications/bulk-delete` ·
-`DELETE /notifications/delete-all` · `GET /webpush/status` ·
-`POST /webpush/subscribe` · `DELETE /webpush/unsubscribe`.
-**Middleware:** notifications routes use `auth:sanctum` + `business.active`;
-web-push routes use `auth:sanctum` only.
-**Notable behavior:** notification types are `business_status`,
-`platform_message`, `user_status`, and pipeline events
-(`pipeline.assignment`, `pipeline.comment`, `pipeline.announcement`,
-`pipeline.poll`, `pipeline.reminder`, `pipeline.board_message`) - the inbox is
-for team messages and pipeline activity, not stock/payment alerts. Opening a
-message auto-marks it read; unread bubbles show on the bell. Web Push is
-browser-only (hidden in Electron) and delivers new orders, sales, and account
-updates as system notifications even while the app is closed. The order sound
-and big-order threshold are device-local preferences for business accounts.
 PUBLISHED TITLE: A chime when the order comes in.
 SHORT-FORM VARIANT: A chime when the order comes in.
 PUBLISHED DESCRIPTION: Set the order sound on Custosell so your device chimes when a new open order arrives - and set a big-order threshold so large orders get an urgent chime and a highlighted alert. Try free #custosell #notifications #webpush #alerts #Custosell #SmallBusiness
@@ -17389,7 +17360,36 @@
   - Screen-record clips: the Screen flow steps, trimmed to the script beats
   - Captions / subtitles: full on-screen captions exported as a caption file
   - Brand overlay / watermark: Custosell logo, corner placement
-  - Music: royalty-free background bed, low volume under the voiceover</t>
+  - Music: royalty-free background bed, low volume under the voiceover
+  - ---
+  - ## Technical reference (source of truth)
+  - **Screens:** `/notifications` [M] (modules/notifications/NotificationsPage) -
+  - inbox with All/Unread filters, open/read, mark-all-read, delete
+  - single/selected/all; the navbar bell (HeaderNotifications) shows the unread
+  - count; PushNotificationsCard and OrderSoundCard live at the top of the inbox.
+  - **User actions (FE hooks):** `useNotifications` (paginated, `per_page`,
+  - `unread_only`) · `useNotificationUnreadCount` · `useMarkNotificationRead` ·
+  - `useMarkAllNotificationsRead` · `useDeleteNotification` ·
+  - `useBulkDeleteNotifications` · `useDeleteAllNotifications` · `useWebPush`
+  - (toggle + status via `fetchWebPushStatus` / `storePushSubscription` /
+  - `removePushSubscription`) · `useSoundPreferences` (`orderSound`,
+  - `bigOrderThreshold`).
+  - **API endpoints (BE):** `GET /notifications` · `GET /notifications/unread-count`
+  - · `PATCH /notifications/read-all` · `PATCH /notifications/{id}/read` ·
+  - `DELETE /notifications/{id}` · `POST /notifications/bulk-delete` ·
+  - `DELETE /notifications/delete-all` · `GET /webpush/status` ·
+  - `POST /webpush/subscribe` · `DELETE /webpush/unsubscribe`.
+  - **Middleware:** notifications routes use `auth:sanctum` + `business.active`;
+  - web-push routes use `auth:sanctum` only.
+  - **Notable behavior:** notification types are `business_status`,
+  - `platform_message`, `user_status`, and pipeline events
+  - (`pipeline.assignment`, `pipeline.comment`, `pipeline.announcement`,
+  - `pipeline.poll`, `pipeline.reminder`, `pipeline.board_message`) - the inbox is
+  - for team messages and pipeline activity, not stock/payment alerts. Opening a
+  - message auto-marks it read; unread bubbles show on the bell. Web Push is
+  - browser-only (hidden in Electron) and delivers new orders, sales, and account
+  - updates as system notifications even while the app is closed. The order sound
+  - and big-order threshold are device-local preferences for business accounts.</t>
         </is>
       </c>
       <c r="D278" s="5" t="n"/>
@@ -17663,27 +17663,6 @@
 DEMO DATA: A notes board with a few notes.
 CTA: Try free
 RELATED: [18-quick-notes.md](./18-quick-notes.md)
----
-## Technical reference (source of truth)
-**Screens:** `/notes` [M] (modules/notes/QuickNotesPage) - sticky-note board with
-search bar, tag chips, New note modal, pin/drag, Background picker, Full screen
-toggle; notes are also reachable from the navbar Quick Notes dropdown.
-**User actions (FE hooks):** `useQuickNotes` · `useCreateQuickNote` ·
-`useUpdateQuickNote` · `useDeleteQuickNote` · `useReorderQuickNotes` ·
-`useRenameQuickNoteTag` · `useRemoveQuickNoteTag` · `useSaveNotesBackground` ·
-`canShareQuickNotes` (business accounts only - personal accounts keep notes
-private).
-**API endpoints (BE):** `GET|POST /quick-notes` · `PUT|PATCH|DELETE
-/quick-notes/{note_id}` · `POST /quick-notes/reorder` ·
-`POST /quick-notes/background` · `POST /quick-notes/tags/rename` ·
-`POST /quick-notes/tags/remove`.
-**Middleware:** `auth:sanctum` + `business.active` + `subscription.active`.
-**Notable behavior:** search and tag filtering are client-side (no search
-endpoint) - the search box filters notes by title/body and tag chips filter the
-board; tag rename/remove are the only tag endpoints. Offline-first: creates,
-updates, and deletes complete locally and sync later (dedupe by `client_uuid`,
-pending-sync badges on notes); `is_shared` notes show a Shared badge plus the
-author's name and are visible to the whole organization.
 PUBLISHED TITLE: Your notes, your style.
 SHORT-FORM VARIANT: Your notes
 PUBLISHED DESCRIPTION: Change the look of your quick notes board on Custosell - pick a background, use full-screen mode to hide navigation, and color-code notes the way you like. Try free #custosell #quicknotes #notes #memo #Custosell #SmallBusiness
@@ -17693,7 +17672,28 @@
   - Screen-record clips: the Screen flow steps, trimmed to the script beats
   - Captions / subtitles: full on-screen captions exported as a caption file
   - Brand overlay / watermark: Custosell logo, corner placement
-  - Music: royalty-free background bed, low volume under the voiceover</t>
+  - Music: royalty-free background bed, low volume under the voiceover
+  - ---
+  - ## Technical reference (source of truth)
+  - **Screens:** `/notes` [M] (modules/notes/QuickNotesPage) - sticky-note board with
+  - search bar, tag chips, New note modal, pin/drag, Background picker, Full screen
+  - toggle; notes are also reachable from the navbar Quick Notes dropdown.
+  - **User actions (FE hooks):** `useQuickNotes` · `useCreateQuickNote` ·
+  - `useUpdateQuickNote` · `useDeleteQuickNote` · `useReorderQuickNotes` ·
+  - `useRenameQuickNoteTag` · `useRemoveQuickNoteTag` · `useSaveNotesBackground` ·
+  - `canShareQuickNotes` (business accounts only - personal accounts keep notes
+  - private).
+  - **API endpoints (BE):** `GET|POST /quick-notes` · `PUT|PATCH|DELETE
+  - /quick-notes/{note_id}` · `POST /quick-notes/reorder` ·
+  - `POST /quick-notes/background` · `POST /quick-notes/tags/rename` ·
+  - `POST /quick-notes/tags/remove`.
+  - **Middleware:** `auth:sanctum` + `business.active` + `subscription.active`.
+  - **Notable behavior:** search and tag filtering are client-side (no search
+  - endpoint) - the search box filters notes by title/body and tag chips filter the
+  - board; tag rename/remove are the only tag endpoints. Offline-first: creates,
+  - updates, and deletes complete locally and sync later (dedupe by `client_uuid`,
+  - pending-sync badges on notes); `is_shared` notes show a Shared badge plus the
+  - author's name and are visible to the whole organization.</t>
         </is>
       </c>
       <c r="D283" s="5" t="n"/>
@@ -17988,35 +17988,6 @@
 contact details.
 CTA: Try free
 RELATED: [22-guide.md](./22-guide.md)
----
-## Technical reference (source of truth)
-**Screens:** `/guide/tutorials` (search + category filter + video cards) ·
-`/guide/faqs` (category accordion + search) · `/guide/feedback` (compose +
-Your submissions with status badges and team replies) · `/guide/contact`
-(support email + phone lines with copy buttons). All under
-`ModuleAccessMiddleware module="guide"`.
-**User actions (FE hooks):** `useGuideTutorials` (GET `/guide/tutorials`) ·
-`useGuideFaqs` (GET `/guide/faqs`) · `usePublicFaqs` (GET `/public/faqs`) ·
-`useMyGuideFeedback` (GET `/guide/feedback/mine`, merged with local pending
-via `readWithOfflineStrategy`) · `useCreateGuideFeedback` (POST
-`/guide/feedback`; offline-first via `completeOfflineGuideFeedbackInstant` -
-queues a mutation and returns a local pending record) ·
-`useDeleteMyGuideFeedback` + `useBulkDeleteMyGuideFeedback` (DELETE
-`/guide/feedback/{id}` / POST `/guide/feedback/bulk-delete`, removing local
-queue entries for unsent items)
-**Feedback status lifecycle:** `submitted` -&gt; `acknowledged` -&gt;
-`in_progress` -&gt; `resolved` / `closed`; staff replies surface on the user's
-submission card; local records carry `_pendingSync` / `_syncFailed` / `_localId`
-markers.
-**API endpoints (BE):** `guide.php` (auth:sanctum + business.active):
-`GET /guide/tutorials` · `GET /guide/faqs` · `GET /guide/feedback/mine` ·
-`POST /guide/feedback` · `POST /guide/feedback/bulk-delete` ·
-`DELETE /guide/feedback/{guideFeedback}` · `public.php`: `GET /public/faqs`
-(no auth)
-**Platform admin (not end-user):** `/platform/guide/*` - manage tutorials
-(create/edit/publish, thumbnail upload + preview) with
-`platform.guide.manage`, manage FAQs, and triage feedback (status updates,
-staff replies, bulk actions) with `platform.guide.feedback.manage`.
 PUBLISHED TITLE: A human, one tap away.
 SHORT-FORM VARIANT: A human
 PUBLISHED DESCRIPTION: Reach the Custosell team when you need a person - support email and phone lines with one-tap copy, plus business hours. Works offline too: the details stay copyable so you can contact the team after you reconnect. Try free #custosell #guide #tutorials #faq #Custosell #SmallBusiness
@@ -18026,7 +17997,36 @@
   - Screen-record clips: the Screen flow steps, trimmed to the script beats
   - Captions / subtitles: full on-screen captions exported as a caption file
   - Brand overlay / watermark: Custosell logo, corner placement
-  - Music: royalty-free background bed, low volume under the voiceover</t>
+  - Music: royalty-free background bed, low volume under the voiceover
+  - ---
+  - ## Technical reference (source of truth)
+  - **Screens:** `/guide/tutorials` (search + category filter + video cards) ·
+  - `/guide/faqs` (category accordion + search) · `/guide/feedback` (compose +
+  - Your submissions with status badges and team replies) · `/guide/contact`
+  - (support email + phone lines with copy buttons). All under
+  - `ModuleAccessMiddleware module="guide"`.
+  - **User actions (FE hooks):** `useGuideTutorials` (GET `/guide/tutorials`) ·
+  - `useGuideFaqs` (GET `/guide/faqs`) · `usePublicFaqs` (GET `/public/faqs`) ·
+  - `useMyGuideFeedback` (GET `/guide/feedback/mine`, merged with local pending
+  - via `readWithOfflineStrategy`) · `useCreateGuideFeedback` (POST
+  - `/guide/feedback`; offline-first via `completeOfflineGuideFeedbackInstant` -
+  - queues a mutation and returns a local pending record) ·
+  - `useDeleteMyGuideFeedback` + `useBulkDeleteMyGuideFeedback` (DELETE
+  - `/guide/feedback/{id}` / POST `/guide/feedback/bulk-delete`, removing local
+  - queue entries for unsent items)
+  - **Feedback status lifecycle:** `submitted` -&gt; `acknowledged` -&gt;
+  - `in_progress` -&gt; `resolved` / `closed`; staff replies surface on the user's
+  - submission card; local records carry `_pendingSync` / `_syncFailed` / `_localId`
+  - markers.
+  - **API endpoints (BE):** `guide.php` (auth:sanctum + business.active):
+  - `GET /guide/tutorials` · `GET /guide/faqs` · `GET /guide/feedback/mine` ·
+  - `POST /guide/feedback` · `POST /guide/feedback/bulk-delete` ·
+  - `DELETE /guide/feedback/{guideFeedback}` · `public.php`: `GET /public/faqs`
+  - (no auth)
+  - **Platform admin (not end-user):** `/platform/guide/*` - manage tutorials
+  - (create/edit/publish, thumbnail upload + preview) with
+  - `platform.guide.manage`, manage FAQs, and triage feedback (status updates,
+  - staff replies, bulk actions) with `platform.guide.feedback.manage`.</t>
         </is>
       </c>
       <c r="D288" s="5" t="n"/>

</xml_diff>